<commit_message>
Working model for IT
</commit_message>
<xml_diff>
--- a/input/policy parameters.xlsx
+++ b/input/policy parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Patryk\git\SimPaths_HU\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B052507F-7339-41BF-A20C-12BAD36711ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0DCCD40-425F-4523-8480-58EEFFD76409}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="3" activeTab="5" xr2:uid="{E29F3EB7-07F0-4B2F-ABCD-03E4363B7DD7}"/>
+    <workbookView xWindow="-83" yWindow="0" windowWidth="14566" windowHeight="17363" firstSheet="2" activeTab="5" xr2:uid="{E29F3EB7-07F0-4B2F-ABCD-03E4363B7DD7}"/>
   </bookViews>
   <sheets>
     <sheet name="disability" sheetId="10" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="43">
   <si>
     <t>CAPITAL LIMITS</t>
   </si>
@@ -174,48 +174,6 @@
   </si>
   <si>
     <t>Share</t>
-  </si>
-  <si>
-    <t>0.582</t>
-  </si>
-  <si>
-    <t>0.586</t>
-  </si>
-  <si>
-    <t>0.5822</t>
-  </si>
-  <si>
-    <t>0.5823</t>
-  </si>
-  <si>
-    <t>0.5805</t>
-  </si>
-  <si>
-    <t>0.5832</t>
-  </si>
-  <si>
-    <t>0.5757</t>
-  </si>
-  <si>
-    <t>0.5647</t>
-  </si>
-  <si>
-    <t>0.5671</t>
-  </si>
-  <si>
-    <t>0.5638</t>
-  </si>
-  <si>
-    <t>0.5653</t>
-  </si>
-  <si>
-    <t>0.5515</t>
-  </si>
-  <si>
-    <t>0.5449</t>
-  </si>
-  <si>
-    <t>0.5513</t>
   </si>
 </sst>
 </file>
@@ -600,7 +558,7 @@
         <v>2010</v>
       </c>
       <c r="B2">
-        <v>0.04</v>
+        <v>9.5999999999999992E-3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.45">
@@ -608,7 +566,7 @@
         <v>2011</v>
       </c>
       <c r="B3">
-        <v>0.04</v>
+        <v>9.5999999999999992E-3</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.45">
@@ -616,7 +574,7 @@
         <v>2012</v>
       </c>
       <c r="B4">
-        <v>3.9199999999999999E-2</v>
+        <v>8.9999999999999993E-3</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.45">
@@ -624,7 +582,7 @@
         <v>2013</v>
       </c>
       <c r="B5">
-        <v>3.7100000000000001E-2</v>
+        <v>8.8000000000000005E-3</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.45">
@@ -632,7 +590,7 @@
         <v>2014</v>
       </c>
       <c r="B6">
-        <v>3.73E-2</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.45">
@@ -640,7 +598,7 @@
         <v>2015</v>
       </c>
       <c r="B7">
-        <v>3.7600000000000001E-2</v>
+        <v>9.7000000000000003E-3</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.45">
@@ -648,7 +606,7 @@
         <v>2016</v>
       </c>
       <c r="B8">
-        <v>3.61E-2</v>
+        <v>7.9000000000000008E-3</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.45">
@@ -656,7 +614,7 @@
         <v>2017</v>
       </c>
       <c r="B9">
-        <v>3.3700000000000001E-2</v>
+        <v>6.1000000000000004E-3</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.45">
@@ -664,7 +622,7 @@
         <v>2018</v>
       </c>
       <c r="B10">
-        <v>2.98E-2</v>
+        <v>6.7000000000000002E-3</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.45">
@@ -672,7 +630,7 @@
         <v>2019</v>
       </c>
       <c r="B11">
-        <v>2.76E-2</v>
+        <v>1.2699999999999999E-2</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.45">
@@ -680,7 +638,7 @@
         <v>2020</v>
       </c>
       <c r="B12">
-        <v>2.76E-2</v>
+        <v>1.24E-2</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.45">
@@ -688,7 +646,7 @@
         <v>2021</v>
       </c>
       <c r="B13">
-        <v>2.9600000000000001E-2</v>
+        <v>1.5599999999999999E-2</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.45">
@@ -696,7 +654,7 @@
         <v>2022</v>
       </c>
       <c r="B14">
-        <v>2.7E-2</v>
+        <v>1.7299999999999999E-2</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.45">
@@ -704,7 +662,7 @@
         <v>2023</v>
       </c>
       <c r="B15">
-        <v>2.6499999999999999E-2</v>
+        <v>1.5599999999999999E-2</v>
       </c>
     </row>
   </sheetData>
@@ -2853,208 +2811,208 @@
       <c r="A2">
         <v>2010</v>
       </c>
-      <c r="B2" t="s">
-        <v>43</v>
+      <c r="B2">
+        <v>0.505</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>2011</v>
       </c>
-      <c r="B3" t="s">
-        <v>44</v>
+      <c r="B3">
+        <v>0.505</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>2012</v>
       </c>
-      <c r="B4" t="s">
-        <v>45</v>
+      <c r="B4">
+        <v>0.50360000000000005</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>2013</v>
       </c>
-      <c r="B5" t="s">
-        <v>46</v>
+      <c r="B5">
+        <v>0.50329999999999997</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>2014</v>
       </c>
-      <c r="B6" t="s">
-        <v>47</v>
+      <c r="B6">
+        <v>0.50080000000000002</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>2015</v>
       </c>
-      <c r="B7" t="s">
-        <v>48</v>
+      <c r="B7">
+        <v>0.50619999999999998</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>2016</v>
       </c>
-      <c r="B8" t="s">
-        <v>49</v>
+      <c r="B8">
+        <v>0.48820000000000002</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>2017</v>
       </c>
-      <c r="B9" t="s">
-        <v>50</v>
+      <c r="B9">
+        <v>0.48010000000000003</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>2018</v>
       </c>
-      <c r="B10" t="s">
-        <v>51</v>
+      <c r="B10">
+        <v>0.47770000000000001</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A11">
         <v>2019</v>
       </c>
-      <c r="B11" t="s">
-        <v>52</v>
+      <c r="B11">
+        <v>0.47460000000000002</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A12">
         <v>2020</v>
       </c>
-      <c r="B12" t="s">
-        <v>53</v>
+      <c r="B12">
+        <v>0.4955</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A13">
         <v>2021</v>
       </c>
-      <c r="B13" t="s">
-        <v>54</v>
+      <c r="B13">
+        <v>0.49049999999999999</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A14">
         <v>2022</v>
       </c>
-      <c r="B14" t="s">
-        <v>55</v>
+      <c r="B14">
+        <v>0.47070000000000001</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A15">
         <v>2023</v>
       </c>
-      <c r="B15" t="s">
-        <v>56</v>
+      <c r="B15">
+        <v>0.47260000000000002</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A16">
         <v>2024</v>
       </c>
-      <c r="B16" t="s">
-        <v>56</v>
+      <c r="B16">
+        <v>0.47260000000000002</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A17">
         <v>2025</v>
       </c>
-      <c r="B17" t="s">
-        <v>56</v>
+      <c r="B17">
+        <v>0.47260000000000002</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A18">
         <v>2026</v>
       </c>
-      <c r="B18" t="s">
-        <v>56</v>
+      <c r="B18">
+        <v>0.47260000000000002</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A19">
         <v>2027</v>
       </c>
-      <c r="B19" t="s">
-        <v>56</v>
+      <c r="B19">
+        <v>0.47260000000000002</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A20">
         <v>2028</v>
       </c>
-      <c r="B20" t="s">
-        <v>56</v>
+      <c r="B20">
+        <v>0.47260000000000002</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A21">
         <v>2029</v>
       </c>
-      <c r="B21" t="s">
-        <v>56</v>
+      <c r="B21">
+        <v>0.47260000000000002</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A22">
         <v>2030</v>
       </c>
-      <c r="B22" t="s">
-        <v>56</v>
+      <c r="B22">
+        <v>0.47260000000000002</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A23">
         <v>2031</v>
       </c>
-      <c r="B23" t="s">
-        <v>56</v>
+      <c r="B23">
+        <v>0.47260000000000002</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A24">
         <v>2032</v>
       </c>
-      <c r="B24" t="s">
-        <v>56</v>
+      <c r="B24">
+        <v>0.47260000000000002</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A25">
         <v>2033</v>
       </c>
-      <c r="B25" t="s">
-        <v>56</v>
+      <c r="B25">
+        <v>0.47260000000000002</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A26">
         <v>2034</v>
       </c>
-      <c r="B26" t="s">
-        <v>56</v>
+      <c r="B26">
+        <v>0.47260000000000002</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A27">
         <v>2035</v>
       </c>
-      <c r="B27" t="s">
-        <v>56</v>
+      <c r="B27">
+        <v>0.47260000000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update partnership alignment targets
-targets were incorrectly specified in relation to the entire population, while alignment was performed on the population of individuals aged 18+. Targets have been updated to represent the 18+ sub-population who can change their cohabitation status.
</commit_message>
<xml_diff>
--- a/input/policy parameters.xlsx
+++ b/input/policy parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Patryk\git\SimPaths_HU\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0DCCD40-425F-4523-8480-58EEFFD76409}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F244F1F-6D5B-44FB-902E-38585F14C04D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-83" yWindow="0" windowWidth="14566" windowHeight="17363" firstSheet="2" activeTab="5" xr2:uid="{E29F3EB7-07F0-4B2F-ABCD-03E4363B7DD7}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" firstSheet="2" activeTab="5" xr2:uid="{E29F3EB7-07F0-4B2F-ABCD-03E4363B7DD7}"/>
   </bookViews>
   <sheets>
     <sheet name="disability" sheetId="10" r:id="rId1"/>
@@ -543,9 +543,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5BE8D09-68C3-47E4-AB1B-09AAE2124BA2}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>41</v>
       </c>
@@ -553,7 +553,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2010</v>
       </c>
@@ -561,7 +561,7 @@
         <v>9.5999999999999992E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2011</v>
       </c>
@@ -569,7 +569,7 @@
         <v>9.5999999999999992E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2012</v>
       </c>
@@ -577,7 +577,7 @@
         <v>8.9999999999999993E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2013</v>
       </c>
@@ -585,7 +585,7 @@
         <v>8.8000000000000005E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2014</v>
       </c>
@@ -593,7 +593,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2015</v>
       </c>
@@ -601,7 +601,7 @@
         <v>9.7000000000000003E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2016</v>
       </c>
@@ -609,7 +609,7 @@
         <v>7.9000000000000008E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2017</v>
       </c>
@@ -617,7 +617,7 @@
         <v>6.1000000000000004E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2018</v>
       </c>
@@ -625,7 +625,7 @@
         <v>6.7000000000000002E-3</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2019</v>
       </c>
@@ -633,7 +633,7 @@
         <v>1.2699999999999999E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2020</v>
       </c>
@@ -641,7 +641,7 @@
         <v>1.24E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2021</v>
       </c>
@@ -649,7 +649,7 @@
         <v>1.5599999999999999E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2022</v>
       </c>
@@ -657,7 +657,7 @@
         <v>1.7299999999999999E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2023</v>
       </c>
@@ -673,9 +673,9 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA85A294-76F0-4023-B97D-1E7832E0E774}">
   <dimension ref="A1:Y33"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>34</v>
       </c>
@@ -686,7 +686,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>1</v>
       </c>
@@ -702,7 +702,7 @@
       <c r="T2" s="2"/>
       <c r="U2" s="2"/>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>2</v>
       </c>
@@ -758,7 +758,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2015</v>
       </c>
@@ -836,7 +836,7 @@
         <v>0.6613654059472992</v>
       </c>
     </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2016</v>
       </c>
@@ -915,7 +915,7 @@
         <v>0.65666662435166534</v>
       </c>
     </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2017</v>
       </c>
@@ -994,7 +994,7 @@
         <v>0.65162882226991414</v>
       </c>
     </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2018</v>
       </c>
@@ -1073,7 +1073,7 @@
         <v>0.64942413470967808</v>
       </c>
     </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2019</v>
       </c>
@@ -1152,7 +1152,7 @@
         <v>0.64547705146902756</v>
       </c>
     </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2020</v>
       </c>
@@ -1231,7 +1231,7 @@
         <v>0.64460168570888343</v>
       </c>
     </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2021</v>
       </c>
@@ -1310,7 +1310,7 @@
         <v>0.64477324955863657</v>
       </c>
     </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2022</v>
       </c>
@@ -1389,7 +1389,7 @@
         <v>0.64570195231543648</v>
       </c>
     </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2023</v>
       </c>
@@ -1468,7 +1468,7 @@
         <v>0.64737782355652385</v>
       </c>
     </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2024</v>
       </c>
@@ -1529,7 +1529,7 @@
         <v>0.64448143654604106</v>
       </c>
     </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2025</v>
       </c>
@@ -1590,7 +1590,7 @@
         <v>0.64389807700679014</v>
       </c>
     </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2026</v>
       </c>
@@ -1651,7 +1651,7 @@
         <v>0.63601678163112885</v>
       </c>
     </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2027</v>
       </c>
@@ -1712,7 +1712,7 @@
         <v>0.63885715724636716</v>
       </c>
     </row>
-    <row r="17" spans="23:25" x14ac:dyDescent="0.45">
+    <row r="17" spans="23:25" x14ac:dyDescent="0.25">
       <c r="W17">
         <f t="shared" si="11"/>
         <v>2007</v>
@@ -1725,7 +1725,7 @@
         <v>0.63970331929393809</v>
       </c>
     </row>
-    <row r="18" spans="23:25" x14ac:dyDescent="0.45">
+    <row r="18" spans="23:25" x14ac:dyDescent="0.25">
       <c r="W18">
         <f t="shared" si="11"/>
         <v>2008</v>
@@ -1738,7 +1738,7 @@
         <v>0.63745385907812036</v>
       </c>
     </row>
-    <row r="19" spans="23:25" x14ac:dyDescent="0.45">
+    <row r="19" spans="23:25" x14ac:dyDescent="0.25">
       <c r="W19">
         <f t="shared" si="11"/>
         <v>2009</v>
@@ -1751,7 +1751,7 @@
         <v>0.64638142900294271</v>
       </c>
     </row>
-    <row r="20" spans="23:25" x14ac:dyDescent="0.45">
+    <row r="20" spans="23:25" x14ac:dyDescent="0.25">
       <c r="W20">
         <f t="shared" si="11"/>
         <v>2010</v>
@@ -1764,7 +1764,7 @@
         <v>0.64291910814000863</v>
       </c>
     </row>
-    <row r="21" spans="23:25" x14ac:dyDescent="0.45">
+    <row r="21" spans="23:25" x14ac:dyDescent="0.25">
       <c r="W21">
         <f t="shared" si="11"/>
         <v>2011</v>
@@ -1777,7 +1777,7 @@
         <v>0.64183543445918845</v>
       </c>
     </row>
-    <row r="22" spans="23:25" x14ac:dyDescent="0.45">
+    <row r="22" spans="23:25" x14ac:dyDescent="0.25">
       <c r="W22">
         <f t="shared" si="11"/>
         <v>2012</v>
@@ -1790,7 +1790,7 @@
         <v>0.64457311813040019</v>
       </c>
     </row>
-    <row r="23" spans="23:25" x14ac:dyDescent="0.45">
+    <row r="23" spans="23:25" x14ac:dyDescent="0.25">
       <c r="W23">
         <f t="shared" si="11"/>
         <v>2013</v>
@@ -1803,7 +1803,7 @@
         <v>0.64501821298769013</v>
       </c>
     </row>
-    <row r="24" spans="23:25" x14ac:dyDescent="0.45">
+    <row r="24" spans="23:25" x14ac:dyDescent="0.25">
       <c r="W24">
         <f t="shared" si="11"/>
         <v>2014</v>
@@ -1816,7 +1816,7 @@
         <v>0.64303300577959377</v>
       </c>
     </row>
-    <row r="25" spans="23:25" x14ac:dyDescent="0.45">
+    <row r="25" spans="23:25" x14ac:dyDescent="0.25">
       <c r="W25">
         <f t="shared" si="11"/>
         <v>2015</v>
@@ -1829,7 +1829,7 @@
         <v>0.64350137796521267</v>
       </c>
     </row>
-    <row r="26" spans="23:25" x14ac:dyDescent="0.45">
+    <row r="26" spans="23:25" x14ac:dyDescent="0.25">
       <c r="W26">
         <f t="shared" si="11"/>
         <v>2016</v>
@@ -1842,7 +1842,7 @@
         <v>0.64443090532156433</v>
       </c>
     </row>
-    <row r="27" spans="23:25" x14ac:dyDescent="0.45">
+    <row r="27" spans="23:25" x14ac:dyDescent="0.25">
       <c r="W27">
         <f t="shared" si="11"/>
         <v>2017</v>
@@ -1855,7 +1855,7 @@
         <v>0.64369538754708922</v>
       </c>
     </row>
-    <row r="28" spans="23:25" x14ac:dyDescent="0.45">
+    <row r="28" spans="23:25" x14ac:dyDescent="0.25">
       <c r="W28">
         <f t="shared" si="11"/>
         <v>2018</v>
@@ -1868,7 +1868,7 @@
         <v>0.64389678969687036</v>
       </c>
     </row>
-    <row r="29" spans="23:25" x14ac:dyDescent="0.45">
+    <row r="29" spans="23:25" x14ac:dyDescent="0.25">
       <c r="W29">
         <f t="shared" si="11"/>
         <v>2019</v>
@@ -1881,7 +1881,7 @@
         <v>0.63975244582712099</v>
       </c>
     </row>
-    <row r="30" spans="23:25" x14ac:dyDescent="0.45">
+    <row r="30" spans="23:25" x14ac:dyDescent="0.25">
       <c r="W30">
         <f t="shared" si="11"/>
         <v>2020</v>
@@ -1894,7 +1894,7 @@
         <v>0.64948824720523413</v>
       </c>
     </row>
-    <row r="31" spans="23:25" x14ac:dyDescent="0.45">
+    <row r="31" spans="23:25" x14ac:dyDescent="0.25">
       <c r="W31">
         <f t="shared" si="11"/>
         <v>2021</v>
@@ -1907,7 +1907,7 @@
         <v>0.64443733677754689</v>
       </c>
     </row>
-    <row r="32" spans="23:25" x14ac:dyDescent="0.45">
+    <row r="32" spans="23:25" x14ac:dyDescent="0.25">
       <c r="W32">
         <v>2022</v>
       </c>
@@ -1916,7 +1916,7 @@
         <v>0.64425404141077236</v>
       </c>
     </row>
-    <row r="33" spans="23:25" x14ac:dyDescent="0.45">
+    <row r="33" spans="23:25" x14ac:dyDescent="0.25">
       <c r="W33">
         <v>2023</v>
       </c>
@@ -1933,13 +1933,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95F81ED4-EE1A-4486-BAEC-BC92A19478AC}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.3984375" customWidth="1"/>
+    <col min="1" max="1" width="13.42578125" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -1947,7 +1947,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1955,7 +1955,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1963,7 +1963,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -1971,7 +1971,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -1982,17 +1982,17 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>37</v>
       </c>
@@ -2008,9 +2008,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5A30919-82CE-4DA6-A5C0-32D0B4E57BD6}">
   <dimension ref="A1:K16"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>23</v>
       </c>
@@ -2039,7 +2039,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2015</v>
       </c>
@@ -2068,7 +2068,7 @@
         <v>23250</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2016</v>
       </c>
@@ -2097,7 +2097,7 @@
         <v>23088.381330685203</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2017</v>
       </c>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="K4" s="1"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2018</v>
       </c>
@@ -2157,7 +2157,7 @@
       </c>
       <c r="K5" s="1"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2019</v>
       </c>
@@ -2187,7 +2187,7 @@
       </c>
       <c r="K6" s="1"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2020</v>
       </c>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="K7" s="1"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2021</v>
       </c>
@@ -2247,7 +2247,7 @@
       </c>
       <c r="K8" s="1"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2022</v>
       </c>
@@ -2277,7 +2277,7 @@
       </c>
       <c r="K9" s="1"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2023</v>
       </c>
@@ -2307,7 +2307,7 @@
       </c>
       <c r="K10" s="1"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2024</v>
       </c>
@@ -2337,7 +2337,7 @@
       </c>
       <c r="K11" s="1"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2025</v>
       </c>
@@ -2367,7 +2367,7 @@
       </c>
       <c r="K12" s="1"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2026</v>
       </c>
@@ -2397,7 +2397,7 @@
       </c>
       <c r="K13" s="1"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2027</v>
       </c>
@@ -2427,10 +2427,10 @@
       </c>
       <c r="K14" s="1"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="K15" s="1"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="K16" s="1"/>
     </row>
   </sheetData>
@@ -2441,9 +2441,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{542CF42B-7BCB-429C-A72F-92D7D9CDCB1D}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>41</v>
       </c>
@@ -2451,7 +2451,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2010</v>
       </c>
@@ -2459,7 +2459,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2011</v>
       </c>
@@ -2467,7 +2467,7 @@
         <v>0.20200000000000001</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2012</v>
       </c>
@@ -2475,7 +2475,7 @@
         <v>0.20300000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2013</v>
       </c>
@@ -2483,7 +2483,7 @@
         <v>0.20599999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2014</v>
       </c>
@@ -2491,7 +2491,7 @@
         <v>0.20699999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2015</v>
       </c>
@@ -2499,7 +2499,7 @@
         <v>0.215</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2016</v>
       </c>
@@ -2507,7 +2507,7 @@
         <v>0.22</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2017</v>
       </c>
@@ -2515,7 +2515,7 @@
         <v>0.23</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2018</v>
       </c>
@@ -2523,7 +2523,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2019</v>
       </c>
@@ -2531,7 +2531,7 @@
         <v>0.26</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2020</v>
       </c>
@@ -2539,7 +2539,7 @@
         <v>0.28000000000000003</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2021</v>
       </c>
@@ -2547,7 +2547,7 @@
         <v>0.28000000000000003</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2022</v>
       </c>
@@ -2555,7 +2555,7 @@
         <v>0.26</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2023</v>
       </c>
@@ -2571,9 +2571,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58D18F52-AE20-431C-A8C1-CEFDA270A8FD}">
   <dimension ref="A1:B27"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>41</v>
       </c>
@@ -2581,7 +2581,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2010</v>
       </c>
@@ -2589,7 +2589,7 @@
         <v>0.23899999999999999</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2011</v>
       </c>
@@ -2597,7 +2597,7 @@
         <v>0.23899999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2012</v>
       </c>
@@ -2605,7 +2605,7 @@
         <v>0.23400000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2013</v>
       </c>
@@ -2613,7 +2613,7 @@
         <v>0.23</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2014</v>
       </c>
@@ -2621,7 +2621,7 @@
         <v>0.22600000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2015</v>
       </c>
@@ -2629,7 +2629,7 @@
         <v>0.219</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2016</v>
       </c>
@@ -2637,7 +2637,7 @@
         <v>0.218</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2017</v>
       </c>
@@ -2645,7 +2645,7 @@
         <v>0.21299999999999999</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2018</v>
       </c>
@@ -2653,7 +2653,7 @@
         <v>0.21</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2019</v>
       </c>
@@ -2661,7 +2661,7 @@
         <v>0.20499999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2020</v>
       </c>
@@ -2669,7 +2669,7 @@
         <v>0.20399999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2021</v>
       </c>
@@ -2677,7 +2677,7 @@
         <v>0.19700000000000001</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2022</v>
       </c>
@@ -2685,7 +2685,7 @@
         <v>0.19500000000000001</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2023</v>
       </c>
@@ -2693,7 +2693,7 @@
         <v>0.188</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2024</v>
       </c>
@@ -2701,7 +2701,7 @@
         <v>0.188</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2025</v>
       </c>
@@ -2709,7 +2709,7 @@
         <v>0.188</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2026</v>
       </c>
@@ -2717,7 +2717,7 @@
         <v>0.188</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2027</v>
       </c>
@@ -2725,7 +2725,7 @@
         <v>0.188</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2028</v>
       </c>
@@ -2733,7 +2733,7 @@
         <v>0.188</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2029</v>
       </c>
@@ -2741,7 +2741,7 @@
         <v>0.188</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2030</v>
       </c>
@@ -2749,7 +2749,7 @@
         <v>0.188</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2031</v>
       </c>
@@ -2757,7 +2757,7 @@
         <v>0.188</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2032</v>
       </c>
@@ -2765,7 +2765,7 @@
         <v>0.188</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2033</v>
       </c>
@@ -2773,7 +2773,7 @@
         <v>0.188</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2034</v>
       </c>
@@ -2781,7 +2781,7 @@
         <v>0.188</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2035</v>
       </c>
@@ -2797,9 +2797,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8252C88-1FFA-4D3B-9F14-2D9286827575}">
   <dimension ref="A1:B27"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>41</v>
       </c>
@@ -2807,212 +2807,212 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2010</v>
       </c>
       <c r="B2">
-        <v>0.505</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+        <v>0.60912390000000005</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2011</v>
       </c>
       <c r="B3">
-        <v>0.505</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+        <v>0.60912390000000005</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2012</v>
       </c>
       <c r="B4">
-        <v>0.50360000000000005</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+        <v>0.60256900000000002</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2013</v>
       </c>
       <c r="B5">
-        <v>0.50329999999999997</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+        <v>0.59983640000000005</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2014</v>
       </c>
       <c r="B6">
-        <v>0.50080000000000002</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+        <v>0.59351379999999998</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2015</v>
       </c>
       <c r="B7">
-        <v>0.50619999999999998</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+        <v>0.6030934</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2016</v>
       </c>
       <c r="B8">
-        <v>0.48820000000000002</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+        <v>0.57539309999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2017</v>
       </c>
       <c r="B9">
-        <v>0.48010000000000003</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+        <v>0.55984630000000002</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2018</v>
       </c>
       <c r="B10">
-        <v>0.47770000000000001</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
+        <v>0.55409109999999995</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2019</v>
       </c>
       <c r="B11">
-        <v>0.47460000000000002</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
+        <v>0.54393720000000001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2020</v>
       </c>
       <c r="B12">
-        <v>0.4955</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.45">
+        <v>0.56667990000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2021</v>
       </c>
       <c r="B13">
-        <v>0.49049999999999999</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
+        <v>0.55765529999999996</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2022</v>
       </c>
       <c r="B14">
-        <v>0.47070000000000001</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.45">
+        <v>0.53449530000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2023</v>
       </c>
       <c r="B15">
-        <v>0.47260000000000002</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.45">
+        <v>0.53523100000000001</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2024</v>
       </c>
       <c r="B16">
-        <v>0.47260000000000002</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
+        <v>0.53523100000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2025</v>
       </c>
       <c r="B17">
-        <v>0.47260000000000002</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
+        <v>0.53523100000000001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2026</v>
       </c>
       <c r="B18">
-        <v>0.47260000000000002</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
+        <v>0.53523100000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2027</v>
       </c>
       <c r="B19">
-        <v>0.47260000000000002</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.45">
+        <v>0.53523100000000001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2028</v>
       </c>
       <c r="B20">
-        <v>0.47260000000000002</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.45">
+        <v>0.53523100000000001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2029</v>
       </c>
       <c r="B21">
-        <v>0.47260000000000002</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.45">
+        <v>0.53523100000000001</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2030</v>
       </c>
       <c r="B22">
-        <v>0.47260000000000002</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.45">
+        <v>0.53523100000000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2031</v>
       </c>
       <c r="B23">
-        <v>0.47260000000000002</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.45">
+        <v>0.53523100000000001</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2032</v>
       </c>
       <c r="B24">
-        <v>0.47260000000000002</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.45">
+        <v>0.53523100000000001</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2033</v>
       </c>
       <c r="B25">
-        <v>0.47260000000000002</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.45">
+        <v>0.53523100000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2034</v>
       </c>
       <c r="B26">
-        <v>0.47260000000000002</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.45">
+        <v>0.53523100000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2035</v>
       </c>
       <c r="B27">
-        <v>0.47260000000000002</v>
+        <v>0.53523100000000001</v>
       </c>
     </row>
   </sheetData>
@@ -3024,9 +3024,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C02B2D7-F4EC-4D40-840B-FB6BA99B9F2B}">
   <dimension ref="A1:B27"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>23</v>
       </c>
@@ -3034,7 +3034,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2010</v>
       </c>
@@ -3042,7 +3042,7 @@
         <v>0.63684130000000005</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2011</v>
       </c>
@@ -3050,7 +3050,7 @@
         <v>0.63684130000000005</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2012</v>
       </c>
@@ -3058,7 +3058,7 @@
         <v>0.63086129999999996</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2013</v>
       </c>
@@ -3066,7 +3066,7 @@
         <v>0.62820810000000005</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2014</v>
       </c>
@@ -3074,7 +3074,7 @@
         <v>0.63444250000000002</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2015</v>
       </c>
@@ -3082,7 +3082,7 @@
         <v>0.64983950000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2016</v>
       </c>
@@ -3090,7 +3090,7 @@
         <v>0.66639119999999996</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2017</v>
       </c>
@@ -3098,7 +3098,7 @@
         <v>0.67221770000000003</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2018</v>
       </c>
@@ -3106,7 +3106,7 @@
         <v>0.67153039999999997</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2019</v>
       </c>
@@ -3114,7 +3114,7 @@
         <v>0.67241660000000003</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2020</v>
       </c>
@@ -3122,7 +3122,7 @@
         <v>0.69137210000000004</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2021</v>
       </c>
@@ -3130,7 +3130,7 @@
         <v>0.703434</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2022</v>
       </c>
@@ -3138,7 +3138,7 @@
         <v>0.70015435151515204</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2023</v>
       </c>
@@ -3146,7 +3146,7 @@
         <v>0.70666020046620004</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2024</v>
       </c>
@@ -3154,7 +3154,7 @@
         <v>0.71316604941724904</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2025</v>
       </c>
@@ -3162,7 +3162,7 @@
         <v>0.71967189836829804</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2026</v>
       </c>
@@ -3170,7 +3170,7 @@
         <v>0.72617774731934703</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2027</v>
       </c>
@@ -3178,7 +3178,7 @@
         <v>0.73268359627039603</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2028</v>
       </c>
@@ -3186,7 +3186,7 @@
         <v>0.73918944522144503</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2029</v>
       </c>
@@ -3194,7 +3194,7 @@
         <v>0.74569529417249403</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2030</v>
       </c>
@@ -3202,7 +3202,7 @@
         <v>0.75220114312354303</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2031</v>
       </c>
@@ -3210,7 +3210,7 @@
         <v>0.75870699207459202</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2032</v>
       </c>
@@ -3218,7 +3218,7 @@
         <v>0.76521284102564102</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2033</v>
       </c>
@@ -3226,7 +3226,7 @@
         <v>0.77171868997669002</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2034</v>
       </c>
@@ -3234,7 +3234,7 @@
         <v>0.77822453892773902</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2035</v>
       </c>
@@ -3250,9 +3250,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2ADCB18-5B9A-4019-89E5-BA38EA9BE54A}">
   <dimension ref="A1:B27"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>23</v>
       </c>
@@ -3260,7 +3260,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2010</v>
       </c>
@@ -3268,7 +3268,7 @@
         <v>0.39854529999999999</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2011</v>
       </c>
@@ -3276,7 +3276,7 @@
         <v>0.39854529999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2012</v>
       </c>
@@ -3284,7 +3284,7 @@
         <v>0.4029663</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2013</v>
       </c>
@@ -3292,7 +3292,7 @@
         <v>0.39655180000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2014</v>
       </c>
@@ -3300,7 +3300,7 @@
         <v>0.4070319</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2015</v>
       </c>
@@ -3308,7 +3308,7 @@
         <v>0.40790100000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2016</v>
       </c>
@@ -3316,7 +3316,7 @@
         <v>0.41726039999999998</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2017</v>
       </c>
@@ -3324,7 +3324,7 @@
         <v>0.42810779999999998</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2018</v>
       </c>
@@ -3332,7 +3332,7 @@
         <v>0.42215740000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2019</v>
       </c>
@@ -3340,7 +3340,7 @@
         <v>0.41901169999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2020</v>
       </c>
@@ -3348,7 +3348,7 @@
         <v>0.42423159999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2021</v>
       </c>
@@ -3356,7 +3356,7 @@
         <v>0.41884729999999998</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2022</v>
       </c>
@@ -3364,7 +3364,7 @@
         <v>0.42949969999999998</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2023</v>
       </c>
@@ -3372,7 +3372,7 @@
         <v>0.43197885000000003</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2024</v>
       </c>
@@ -3380,7 +3380,7 @@
         <v>0.4346719</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2025</v>
       </c>
@@ -3388,7 +3388,7 @@
         <v>0.43736494999999997</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2026</v>
       </c>
@@ -3396,7 +3396,7 @@
         <v>0.440058</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2027</v>
       </c>
@@ -3404,7 +3404,7 @@
         <v>0.44275104999999998</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2028</v>
       </c>
@@ -3412,7 +3412,7 @@
         <v>0.44544410000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2029</v>
       </c>
@@ -3420,7 +3420,7 @@
         <v>0.44813714999999998</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2030</v>
       </c>
@@ -3428,7 +3428,7 @@
         <v>0.45083020000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2031</v>
       </c>
@@ -3436,7 +3436,7 @@
         <v>0.45352324999999999</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2032</v>
       </c>
@@ -3444,7 +3444,7 @@
         <v>0.45621630000000002</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2033</v>
       </c>
@@ -3452,7 +3452,7 @@
         <v>0.45890934999999999</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2034</v>
       </c>
@@ -3460,7 +3460,7 @@
         <v>0.46160240000000002</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2035</v>
       </c>
@@ -3476,9 +3476,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D244153-91CD-4DE3-A3BE-886BB7506357}">
   <dimension ref="A1:B27"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>23</v>
       </c>
@@ -3486,7 +3486,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2010</v>
       </c>
@@ -3494,7 +3494,7 @@
         <v>0.7511234</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2011</v>
       </c>
@@ -3502,7 +3502,7 @@
         <v>0.7511234</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2012</v>
       </c>
@@ -3510,7 +3510,7 @@
         <v>0.74668140000000005</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2013</v>
       </c>
@@ -3518,7 +3518,7 @@
         <v>0.74351520000000004</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2014</v>
       </c>
@@ -3526,7 +3526,7 @@
         <v>0.74422900000000003</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2015</v>
       </c>
@@ -3534,7 +3534,7 @@
         <v>0.73707429999999996</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2016</v>
       </c>
@@ -3542,7 +3542,7 @@
         <v>0.74269050000000003</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2017</v>
       </c>
@@ -3550,7 +3550,7 @@
         <v>0.74164249999999998</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2018</v>
       </c>
@@ -3558,7 +3558,7 @@
         <v>0.73936999999999997</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2019</v>
       </c>
@@ -3566,7 +3566,7 @@
         <v>0.7404522</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2020</v>
       </c>
@@ -3574,7 +3574,7 @@
         <v>0.73668559333333306</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2021</v>
       </c>
@@ -3582,7 +3582,7 @@
         <v>0.73539384848484901</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2022</v>
       </c>
@@ -3590,7 +3590,7 @@
         <v>0.73410210363636397</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2023</v>
       </c>
@@ -3598,7 +3598,7 @@
         <v>0.73281035878787903</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2024</v>
       </c>
@@ -3606,7 +3606,7 @@
         <v>0.73151861393939399</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2025</v>
       </c>
@@ -3614,7 +3614,7 @@
         <v>0.73022686909090895</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2026</v>
       </c>
@@ -3622,7 +3622,7 @@
         <v>0.72893512424242402</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2027</v>
       </c>
@@ -3630,7 +3630,7 @@
         <v>0.72764337939393897</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2028</v>
       </c>
@@ -3638,7 +3638,7 @@
         <v>0.72635163454545504</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2029</v>
       </c>
@@ -3646,7 +3646,7 @@
         <v>0.72505988969696999</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2030</v>
       </c>
@@ -3654,7 +3654,7 @@
         <v>0.72376814484848495</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2031</v>
       </c>
@@ -3662,7 +3662,7 @@
         <v>0.72247640000000002</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2032</v>
       </c>
@@ -3670,7 +3670,7 @@
         <v>0.72247640000000002</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2033</v>
       </c>
@@ -3678,7 +3678,7 @@
         <v>0.72247640000000002</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2034</v>
       </c>
@@ -3686,7 +3686,7 @@
         <v>0.72247640000000002</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2035</v>
       </c>

</xml_diff>

<commit_message>
Introduce revised activity status alignment procedure
</commit_message>
<xml_diff>
--- a/input/policy parameters.xlsx
+++ b/input/policy parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Patryk\git\SimPaths_HU\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F244F1F-6D5B-44FB-902E-38585F14C04D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88BA3949-4876-4934-919D-2B43C2A13D68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" firstSheet="2" activeTab="5" xr2:uid="{E29F3EB7-07F0-4B2F-ABCD-03E4363B7DD7}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" firstSheet="5" activeTab="8" xr2:uid="{E29F3EB7-07F0-4B2F-ABCD-03E4363B7DD7}"/>
   </bookViews>
   <sheets>
     <sheet name="disability" sheetId="10" r:id="rId1"/>
@@ -3039,7 +3039,7 @@
         <v>2010</v>
       </c>
       <c r="B2">
-        <v>0.63684130000000005</v>
+        <v>0.49449700000000002</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -3047,7 +3047,7 @@
         <v>2011</v>
       </c>
       <c r="B3">
-        <v>0.63684130000000005</v>
+        <v>0.29497800000000002</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3055,7 +3055,7 @@
         <v>2012</v>
       </c>
       <c r="B4">
-        <v>0.63086129999999996</v>
+        <v>0.30293399999999998</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -3063,7 +3063,7 @@
         <v>2013</v>
       </c>
       <c r="B5">
-        <v>0.62820810000000005</v>
+        <v>0.30091099999999998</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -3071,7 +3071,7 @@
         <v>2014</v>
       </c>
       <c r="B6">
-        <v>0.63444250000000002</v>
+        <v>0.29651699999999998</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -3079,7 +3079,7 @@
         <v>2015</v>
       </c>
       <c r="B7">
-        <v>0.64983950000000001</v>
+        <v>0.30839499999999997</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -3087,7 +3087,7 @@
         <v>2016</v>
       </c>
       <c r="B8">
-        <v>0.66639119999999996</v>
+        <v>0.31296000000000002</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -3095,7 +3095,7 @@
         <v>2017</v>
       </c>
       <c r="B9">
-        <v>0.67221770000000003</v>
+        <v>0.33508500000000002</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -3103,7 +3103,7 @@
         <v>2018</v>
       </c>
       <c r="B10">
-        <v>0.67153039999999997</v>
+        <v>0.36758299999999999</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -3111,7 +3111,7 @@
         <v>2019</v>
       </c>
       <c r="B11">
-        <v>0.67241660000000003</v>
+        <v>0.38047399999999998</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -3119,7 +3119,7 @@
         <v>2020</v>
       </c>
       <c r="B12">
-        <v>0.69137210000000004</v>
+        <v>0.32200600000000001</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -3127,7 +3127,7 @@
         <v>2021</v>
       </c>
       <c r="B13">
-        <v>0.703434</v>
+        <v>0.319162</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -3135,7 +3135,7 @@
         <v>2022</v>
       </c>
       <c r="B14">
-        <v>0.70015435151515204</v>
+        <v>0.31869500000000001</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -3143,7 +3143,7 @@
         <v>2023</v>
       </c>
       <c r="B15">
-        <v>0.70666020046620004</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -3151,7 +3151,7 @@
         <v>2024</v>
       </c>
       <c r="B16">
-        <v>0.71316604941724904</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -3159,7 +3159,7 @@
         <v>2025</v>
       </c>
       <c r="B17">
-        <v>0.71967189836829804</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -3167,7 +3167,7 @@
         <v>2026</v>
       </c>
       <c r="B18">
-        <v>0.72617774731934703</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -3175,7 +3175,7 @@
         <v>2027</v>
       </c>
       <c r="B19">
-        <v>0.73268359627039603</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -3183,7 +3183,7 @@
         <v>2028</v>
       </c>
       <c r="B20">
-        <v>0.73918944522144503</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -3191,7 +3191,7 @@
         <v>2029</v>
       </c>
       <c r="B21">
-        <v>0.74569529417249403</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -3199,7 +3199,7 @@
         <v>2030</v>
       </c>
       <c r="B22">
-        <v>0.75220114312354303</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -3207,7 +3207,7 @@
         <v>2031</v>
       </c>
       <c r="B23">
-        <v>0.75870699207459202</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -3215,7 +3215,7 @@
         <v>2032</v>
       </c>
       <c r="B24">
-        <v>0.76521284102564102</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -3223,7 +3223,7 @@
         <v>2033</v>
       </c>
       <c r="B25">
-        <v>0.77171868997669002</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -3231,7 +3231,7 @@
         <v>2034</v>
       </c>
       <c r="B26">
-        <v>0.77822453892773902</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -3239,7 +3239,7 @@
         <v>2035</v>
       </c>
       <c r="B27">
-        <v>0.78473038787878802</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
   </sheetData>
@@ -3265,7 +3265,7 @@
         <v>2010</v>
       </c>
       <c r="B2">
-        <v>0.39854529999999999</v>
+        <v>0.29497800000000002</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -3273,7 +3273,7 @@
         <v>2011</v>
       </c>
       <c r="B3">
-        <v>0.39854529999999999</v>
+        <v>0.30293399999999998</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3281,7 +3281,7 @@
         <v>2012</v>
       </c>
       <c r="B4">
-        <v>0.4029663</v>
+        <v>0.30091099999999998</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -3289,7 +3289,7 @@
         <v>2013</v>
       </c>
       <c r="B5">
-        <v>0.39655180000000001</v>
+        <v>0.29651699999999998</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -3297,7 +3297,7 @@
         <v>2014</v>
       </c>
       <c r="B6">
-        <v>0.4070319</v>
+        <v>0.30839499999999997</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -3305,7 +3305,7 @@
         <v>2015</v>
       </c>
       <c r="B7">
-        <v>0.40790100000000001</v>
+        <v>0.31296000000000002</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -3313,7 +3313,7 @@
         <v>2016</v>
       </c>
       <c r="B8">
-        <v>0.41726039999999998</v>
+        <v>0.33508500000000002</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -3321,7 +3321,7 @@
         <v>2017</v>
       </c>
       <c r="B9">
-        <v>0.42810779999999998</v>
+        <v>0.36758299999999999</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -3329,7 +3329,7 @@
         <v>2018</v>
       </c>
       <c r="B10">
-        <v>0.42215740000000002</v>
+        <v>0.38047399999999998</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -3337,7 +3337,7 @@
         <v>2019</v>
       </c>
       <c r="B11">
-        <v>0.41901169999999999</v>
+        <v>0.32200600000000001</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -3345,7 +3345,7 @@
         <v>2020</v>
       </c>
       <c r="B12">
-        <v>0.42423159999999999</v>
+        <v>0.319162</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -3353,7 +3353,7 @@
         <v>2021</v>
       </c>
       <c r="B13">
-        <v>0.41884729999999998</v>
+        <v>0.31869500000000001</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -3361,7 +3361,7 @@
         <v>2022</v>
       </c>
       <c r="B14">
-        <v>0.42949969999999998</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -3369,7 +3369,7 @@
         <v>2023</v>
       </c>
       <c r="B15">
-        <v>0.43197885000000003</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -3377,7 +3377,7 @@
         <v>2024</v>
       </c>
       <c r="B16">
-        <v>0.4346719</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -3385,7 +3385,7 @@
         <v>2025</v>
       </c>
       <c r="B17">
-        <v>0.43736494999999997</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -3393,7 +3393,7 @@
         <v>2026</v>
       </c>
       <c r="B18">
-        <v>0.440058</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -3401,7 +3401,7 @@
         <v>2027</v>
       </c>
       <c r="B19">
-        <v>0.44275104999999998</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -3409,7 +3409,7 @@
         <v>2028</v>
       </c>
       <c r="B20">
-        <v>0.44544410000000001</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -3417,7 +3417,7 @@
         <v>2029</v>
       </c>
       <c r="B21">
-        <v>0.44813714999999998</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -3425,7 +3425,7 @@
         <v>2030</v>
       </c>
       <c r="B22">
-        <v>0.45083020000000001</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -3433,7 +3433,7 @@
         <v>2031</v>
       </c>
       <c r="B23">
-        <v>0.45352324999999999</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -3441,7 +3441,7 @@
         <v>2032</v>
       </c>
       <c r="B24">
-        <v>0.45621630000000002</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -3449,7 +3449,7 @@
         <v>2033</v>
       </c>
       <c r="B25">
-        <v>0.45890934999999999</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -3457,7 +3457,7 @@
         <v>2034</v>
       </c>
       <c r="B26">
-        <v>0.46160240000000002</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -3465,7 +3465,7 @@
         <v>2035</v>
       </c>
       <c r="B27">
-        <v>0.46429545</v>
+        <v>0.33229500000000001</v>
       </c>
     </row>
   </sheetData>
@@ -3491,7 +3491,7 @@
         <v>2010</v>
       </c>
       <c r="B2">
-        <v>0.7511234</v>
+        <v>0.62630600000000003</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -3499,7 +3499,7 @@
         <v>2011</v>
       </c>
       <c r="B3">
-        <v>0.7511234</v>
+        <v>0.62630600000000003</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3507,7 +3507,7 @@
         <v>2012</v>
       </c>
       <c r="B4">
-        <v>0.74668140000000005</v>
+        <v>0.61981799999999998</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -3515,7 +3515,7 @@
         <v>2013</v>
       </c>
       <c r="B5">
-        <v>0.74351520000000004</v>
+        <v>0.62006399999999995</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -3523,7 +3523,7 @@
         <v>2014</v>
       </c>
       <c r="B6">
-        <v>0.74422900000000003</v>
+        <v>0.62284799999999996</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -3531,7 +3531,7 @@
         <v>2015</v>
       </c>
       <c r="B7">
-        <v>0.73707429999999996</v>
+        <v>0.63151900000000005</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -3539,7 +3539,7 @@
         <v>2016</v>
       </c>
       <c r="B8">
-        <v>0.74269050000000003</v>
+        <v>0.62040200000000001</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -3547,7 +3547,7 @@
         <v>2017</v>
       </c>
       <c r="B9">
-        <v>0.74164249999999998</v>
+        <v>0.60854799999999998</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -3555,7 +3555,7 @@
         <v>2018</v>
       </c>
       <c r="B10">
-        <v>0.73936999999999997</v>
+        <v>0.60442799999999997</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -3563,7 +3563,7 @@
         <v>2019</v>
       </c>
       <c r="B11">
-        <v>0.7404522</v>
+        <v>0.57280399999999998</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -3571,7 +3571,7 @@
         <v>2020</v>
       </c>
       <c r="B12">
-        <v>0.73668559333333306</v>
+        <v>0.51707499999999995</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -3579,7 +3579,7 @@
         <v>2021</v>
       </c>
       <c r="B13">
-        <v>0.73539384848484901</v>
+        <v>0.54910899999999996</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -3587,7 +3587,7 @@
         <v>2022</v>
       </c>
       <c r="B14">
-        <v>0.73410210363636397</v>
+        <v>0.54368700000000003</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -3595,7 +3595,7 @@
         <v>2023</v>
       </c>
       <c r="B15">
-        <v>0.73281035878787903</v>
+        <v>0.55044300000000002</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -3603,7 +3603,7 @@
         <v>2024</v>
       </c>
       <c r="B16">
-        <v>0.73151861393939399</v>
+        <v>0.55044300000000002</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -3611,7 +3611,7 @@
         <v>2025</v>
       </c>
       <c r="B17">
-        <v>0.73022686909090895</v>
+        <v>0.55044300000000002</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -3619,7 +3619,7 @@
         <v>2026</v>
       </c>
       <c r="B18">
-        <v>0.72893512424242402</v>
+        <v>0.55044300000000002</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -3627,7 +3627,7 @@
         <v>2027</v>
       </c>
       <c r="B19">
-        <v>0.72764337939393897</v>
+        <v>0.55044300000000002</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -3635,7 +3635,7 @@
         <v>2028</v>
       </c>
       <c r="B20">
-        <v>0.72635163454545504</v>
+        <v>0.55044300000000002</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -3643,7 +3643,7 @@
         <v>2029</v>
       </c>
       <c r="B21">
-        <v>0.72505988969696999</v>
+        <v>0.55044300000000002</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -3651,7 +3651,7 @@
         <v>2030</v>
       </c>
       <c r="B22">
-        <v>0.72376814484848495</v>
+        <v>0.55044300000000002</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -3659,7 +3659,7 @@
         <v>2031</v>
       </c>
       <c r="B23">
-        <v>0.72247640000000002</v>
+        <v>0.55044300000000002</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -3667,7 +3667,7 @@
         <v>2032</v>
       </c>
       <c r="B24">
-        <v>0.72247640000000002</v>
+        <v>0.55044300000000002</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -3675,7 +3675,7 @@
         <v>2033</v>
       </c>
       <c r="B25">
-        <v>0.72247640000000002</v>
+        <v>0.55044300000000002</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -3683,7 +3683,7 @@
         <v>2034</v>
       </c>
       <c r="B26">
-        <v>0.72247640000000002</v>
+        <v>0.55044300000000002</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -3691,7 +3691,7 @@
         <v>2035</v>
       </c>
       <c r="B27">
-        <v>0.72247640000000002</v>
+        <v>0.55044300000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update activity alignment targets
-now for seven subgroups matching the labour supply model categories
</commit_message>
<xml_diff>
--- a/input/policy parameters.xlsx
+++ b/input/policy parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Patryk\git\SimPaths_HU\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3410F6B-052D-452F-8F62-CD74EEC8D3D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB338366-4843-4835-8D77-7D3E3B4ECC87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="4" activeTab="11" xr2:uid="{E29F3EB7-07F0-4B2F-ABCD-03E4363B7DD7}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" firstSheet="10" activeTab="12" xr2:uid="{E29F3EB7-07F0-4B2F-ABCD-03E4363B7DD7}"/>
   </bookViews>
   <sheets>
     <sheet name="info" sheetId="2" r:id="rId1"/>
@@ -637,7 +637,7 @@
         <v>2010</v>
       </c>
       <c r="B2">
-        <v>0.60160000000000002</v>
+        <v>0.29414899999999999</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -645,7 +645,7 @@
         <v>2011</v>
       </c>
       <c r="B3">
-        <v>0.60160000000000002</v>
+        <v>0.29414899999999999</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -653,7 +653,7 @@
         <v>2012</v>
       </c>
       <c r="B4">
-        <v>0.57340000000000002</v>
+        <v>0.27185799999999999</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -661,7 +661,7 @@
         <v>2013</v>
       </c>
       <c r="B5">
-        <v>0.53339999999999999</v>
+        <v>0.24763199999999999</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -669,7 +669,7 @@
         <v>2014</v>
       </c>
       <c r="B6">
-        <v>0.54020000000000001</v>
+        <v>0.22253700000000001</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -677,7 +677,7 @@
         <v>2015</v>
       </c>
       <c r="B7">
-        <v>0.54900000000000004</v>
+        <v>0.22546099999999999</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -685,7 +685,7 @@
         <v>2016</v>
       </c>
       <c r="B8">
-        <v>0.56499999999999995</v>
+        <v>0.24279899999999999</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -693,7 +693,7 @@
         <v>2017</v>
       </c>
       <c r="B9">
-        <v>0.58340000000000003</v>
+        <v>0.24468000000000001</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -701,7 +701,7 @@
         <v>2018</v>
       </c>
       <c r="B10">
-        <v>0.60089999999999999</v>
+        <v>0.27390300000000001</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -709,7 +709,7 @@
         <v>2019</v>
       </c>
       <c r="B11">
-        <v>0.61199999999999999</v>
+        <v>0.313029</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -717,7 +717,7 @@
         <v>2020</v>
       </c>
       <c r="B12">
-        <v>0.59789999999999999</v>
+        <v>0.28016600000000003</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -725,7 +725,7 @@
         <v>2021</v>
       </c>
       <c r="B13">
-        <v>0.61580000000000001</v>
+        <v>0.27554800000000002</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -733,7 +733,7 @@
         <v>2022</v>
       </c>
       <c r="B14">
-        <v>0.64449999999999996</v>
+        <v>0.33879599999999999</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -741,7 +741,7 @@
         <v>2023</v>
       </c>
       <c r="B15">
-        <v>0.65080000000000005</v>
+        <v>0.32312099999999999</v>
       </c>
     </row>
   </sheetData>
@@ -767,7 +767,7 @@
         <v>2010</v>
       </c>
       <c r="B2">
-        <v>0.60160000000000002</v>
+        <v>0.84780199999999994</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -775,7 +775,7 @@
         <v>2011</v>
       </c>
       <c r="B3">
-        <v>0.60160000000000002</v>
+        <v>0.84780199999999994</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -783,7 +783,7 @@
         <v>2012</v>
       </c>
       <c r="B4">
-        <v>0.57340000000000002</v>
+        <v>0.80887100000000001</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -791,7 +791,7 @@
         <v>2013</v>
       </c>
       <c r="B5">
-        <v>0.53339999999999999</v>
+        <v>0.77573499999999995</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -799,7 +799,7 @@
         <v>2014</v>
       </c>
       <c r="B6">
-        <v>0.54020000000000001</v>
+        <v>0.75251699999999999</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -807,7 +807,7 @@
         <v>2015</v>
       </c>
       <c r="B7">
-        <v>0.54900000000000004</v>
+        <v>0.75262899999999999</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -815,7 +815,7 @@
         <v>2016</v>
       </c>
       <c r="B8">
-        <v>0.56499999999999995</v>
+        <v>0.75889499999999999</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -823,7 +823,7 @@
         <v>2017</v>
       </c>
       <c r="B9">
-        <v>0.58340000000000003</v>
+        <v>0.79421600000000003</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -831,7 +831,7 @@
         <v>2018</v>
       </c>
       <c r="B10">
-        <v>0.60089999999999999</v>
+        <v>0.78493500000000005</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -839,7 +839,7 @@
         <v>2019</v>
       </c>
       <c r="B11">
-        <v>0.61199999999999999</v>
+        <v>0.83127399999999996</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -847,7 +847,7 @@
         <v>2020</v>
       </c>
       <c r="B12">
-        <v>0.59789999999999999</v>
+        <v>0.88571599999999995</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -855,7 +855,7 @@
         <v>2021</v>
       </c>
       <c r="B13">
-        <v>0.61580000000000001</v>
+        <v>0.84921800000000003</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -863,7 +863,7 @@
         <v>2022</v>
       </c>
       <c r="B14">
-        <v>0.64449999999999996</v>
+        <v>0.89088400000000001</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -871,7 +871,7 @@
         <v>2023</v>
       </c>
       <c r="B15">
-        <v>0.65080000000000005</v>
+        <v>0.78691500000000003</v>
       </c>
     </row>
   </sheetData>
@@ -897,7 +897,7 @@
         <v>2010</v>
       </c>
       <c r="B2">
-        <v>0.60160000000000002</v>
+        <v>0.26522800000000002</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -905,7 +905,7 @@
         <v>2011</v>
       </c>
       <c r="B3">
-        <v>0.60160000000000002</v>
+        <v>0.26522800000000002</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -913,7 +913,7 @@
         <v>2012</v>
       </c>
       <c r="B4">
-        <v>0.57340000000000002</v>
+        <v>0.27356799999999998</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -921,7 +921,7 @@
         <v>2013</v>
       </c>
       <c r="B5">
-        <v>0.53339999999999999</v>
+        <v>0.273926</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -929,7 +929,7 @@
         <v>2014</v>
       </c>
       <c r="B6">
-        <v>0.54020000000000001</v>
+        <v>0.23652200000000001</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -937,7 +937,7 @@
         <v>2015</v>
       </c>
       <c r="B7">
-        <v>0.54900000000000004</v>
+        <v>0.25017800000000001</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -945,7 +945,7 @@
         <v>2016</v>
       </c>
       <c r="B8">
-        <v>0.56499999999999995</v>
+        <v>0.24973799999999999</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -953,7 +953,7 @@
         <v>2017</v>
       </c>
       <c r="B9">
-        <v>0.58340000000000003</v>
+        <v>0.26674399999999998</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -961,7 +961,7 @@
         <v>2018</v>
       </c>
       <c r="B10">
-        <v>0.60089999999999999</v>
+        <v>0.27819100000000002</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -969,7 +969,7 @@
         <v>2019</v>
       </c>
       <c r="B11">
-        <v>0.61199999999999999</v>
+        <v>0.29665599999999998</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -977,7 +977,7 @@
         <v>2020</v>
       </c>
       <c r="B12">
-        <v>0.59789999999999999</v>
+        <v>0.30199500000000001</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -985,7 +985,7 @@
         <v>2021</v>
       </c>
       <c r="B13">
-        <v>0.61580000000000001</v>
+        <v>0.32094800000000001</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -993,7 +993,7 @@
         <v>2022</v>
       </c>
       <c r="B14">
-        <v>0.64449999999999996</v>
+        <v>0.34444900000000001</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -1001,7 +1001,7 @@
         <v>2023</v>
       </c>
       <c r="B15">
-        <v>0.65080000000000005</v>
+        <v>0.37901499999999999</v>
       </c>
     </row>
   </sheetData>
@@ -1027,7 +1027,7 @@
         <v>2010</v>
       </c>
       <c r="B2">
-        <v>0.6119</v>
+        <v>0.92523500000000003</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1035,7 +1035,7 @@
         <v>2011</v>
       </c>
       <c r="B3">
-        <v>0.6119</v>
+        <v>0.92523500000000003</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1043,7 +1043,7 @@
         <v>2012</v>
       </c>
       <c r="B4">
-        <v>0.60709999999999997</v>
+        <v>0.90744100000000005</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1051,7 +1051,7 @@
         <v>2013</v>
       </c>
       <c r="B5">
-        <v>0.59409999999999996</v>
+        <v>0.88748300000000002</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1059,7 +1059,7 @@
         <v>2014</v>
       </c>
       <c r="B6">
-        <v>0.57420000000000004</v>
+        <v>0.89144000000000001</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -1067,7 +1067,7 @@
         <v>2015</v>
       </c>
       <c r="B7">
-        <v>0.58260000000000001</v>
+        <v>0.91203199999999995</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -1075,7 +1075,7 @@
         <v>2016</v>
       </c>
       <c r="B8">
-        <v>0.59130000000000005</v>
+        <v>0.91222300000000001</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1083,7 +1083,7 @@
         <v>2017</v>
       </c>
       <c r="B9">
-        <v>0.61050000000000004</v>
+        <v>0.92773099999999997</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -1091,7 +1091,7 @@
         <v>2018</v>
       </c>
       <c r="B10">
-        <v>0.60829999999999995</v>
+        <v>0.92655100000000001</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -1099,7 +1099,7 @@
         <v>2019</v>
       </c>
       <c r="B11">
-        <v>0.61729999999999996</v>
+        <v>0.94273300000000004</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -1107,7 +1107,7 @@
         <v>2020</v>
       </c>
       <c r="B12">
-        <v>0.63039999999999996</v>
+        <v>0.93638600000000005</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -1115,7 +1115,7 @@
         <v>2021</v>
       </c>
       <c r="B13">
-        <v>0.63660000000000005</v>
+        <v>0.93873399999999996</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -1123,7 +1123,7 @@
         <v>2022</v>
       </c>
       <c r="B14">
-        <v>0.65169999999999995</v>
+        <v>0.95450699999999999</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -1131,7 +1131,7 @@
         <v>2023</v>
       </c>
       <c r="B15">
-        <v>0.65510000000000002</v>
+        <v>0.958484</v>
       </c>
     </row>
   </sheetData>
@@ -3563,7 +3563,7 @@
         <v>2010</v>
       </c>
       <c r="B2">
-        <v>0.60160000000000002</v>
+        <v>0.70775399999999999</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -3571,7 +3571,7 @@
         <v>2011</v>
       </c>
       <c r="B3">
-        <v>0.60160000000000002</v>
+        <v>0.70775399999999999</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3579,7 +3579,7 @@
         <v>2012</v>
       </c>
       <c r="B4">
-        <v>0.57340000000000002</v>
+        <v>0.68374000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -3587,7 +3587,7 @@
         <v>2013</v>
       </c>
       <c r="B5">
-        <v>0.53339999999999999</v>
+        <v>0.64686200000000005</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -3595,7 +3595,7 @@
         <v>2014</v>
       </c>
       <c r="B6">
-        <v>0.54020000000000001</v>
+        <v>0.64708299999999996</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -3603,7 +3603,7 @@
         <v>2015</v>
       </c>
       <c r="B7">
-        <v>0.54900000000000004</v>
+        <v>0.64515100000000003</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -3611,7 +3611,7 @@
         <v>2016</v>
       </c>
       <c r="B8">
-        <v>0.56499999999999995</v>
+        <v>0.66195099999999996</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -3619,7 +3619,7 @@
         <v>2017</v>
       </c>
       <c r="B9">
-        <v>0.58340000000000003</v>
+        <v>0.67321299999999995</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -3627,7 +3627,7 @@
         <v>2018</v>
       </c>
       <c r="B10">
-        <v>0.60089999999999999</v>
+        <v>0.68717399999999995</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -3635,7 +3635,7 @@
         <v>2019</v>
       </c>
       <c r="B11">
-        <v>0.61199999999999999</v>
+        <v>0.698577</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -3643,7 +3643,7 @@
         <v>2020</v>
       </c>
       <c r="B12">
-        <v>0.59789999999999999</v>
+        <v>0.705511</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -3651,7 +3651,7 @@
         <v>2021</v>
       </c>
       <c r="B13">
-        <v>0.61580000000000001</v>
+        <v>0.72767700000000002</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -3659,7 +3659,7 @@
         <v>2022</v>
       </c>
       <c r="B14">
-        <v>0.64449999999999996</v>
+        <v>0.74404400000000004</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -3667,7 +3667,7 @@
         <v>2023</v>
       </c>
       <c r="B15">
-        <v>0.65080000000000005</v>
+        <v>0.75032299999999996</v>
       </c>
     </row>
   </sheetData>
@@ -3693,7 +3693,7 @@
         <v>2010</v>
       </c>
       <c r="B2">
-        <v>0.60160000000000002</v>
+        <v>0.349132</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -3701,7 +3701,7 @@
         <v>2011</v>
       </c>
       <c r="B3">
-        <v>0.60160000000000002</v>
+        <v>0.349132</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3709,7 +3709,7 @@
         <v>2012</v>
       </c>
       <c r="B4">
-        <v>0.57340000000000002</v>
+        <v>0.349132</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -3717,7 +3717,7 @@
         <v>2013</v>
       </c>
       <c r="B5">
-        <v>0.53339999999999999</v>
+        <v>0.30974299999999999</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -3725,7 +3725,7 @@
         <v>2014</v>
       </c>
       <c r="B6">
-        <v>0.54020000000000001</v>
+        <v>0.25676199999999999</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -3733,7 +3733,7 @@
         <v>2015</v>
       </c>
       <c r="B7">
-        <v>0.54900000000000004</v>
+        <v>0.26411699999999999</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -3741,7 +3741,7 @@
         <v>2016</v>
       </c>
       <c r="B8">
-        <v>0.56499999999999995</v>
+        <v>0.27359499999999998</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -3749,7 +3749,7 @@
         <v>2017</v>
       </c>
       <c r="B9">
-        <v>0.58340000000000003</v>
+        <v>0.27618300000000001</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -3757,7 +3757,7 @@
         <v>2018</v>
       </c>
       <c r="B10">
-        <v>0.60089999999999999</v>
+        <v>0.30072199999999999</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -3765,7 +3765,7 @@
         <v>2019</v>
       </c>
       <c r="B11">
-        <v>0.61199999999999999</v>
+        <v>0.32430500000000001</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -3773,7 +3773,7 @@
         <v>2020</v>
       </c>
       <c r="B12">
-        <v>0.59789999999999999</v>
+        <v>0.351267</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -3781,7 +3781,7 @@
         <v>2021</v>
       </c>
       <c r="B13">
-        <v>0.61580000000000001</v>
+        <v>0.26828200000000002</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -3789,7 +3789,7 @@
         <v>2022</v>
       </c>
       <c r="B14">
-        <v>0.64449999999999996</v>
+        <v>0.31243900000000002</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -3797,7 +3797,7 @@
         <v>2023</v>
       </c>
       <c r="B15">
-        <v>0.65080000000000005</v>
+        <v>0.36913600000000002</v>
       </c>
     </row>
   </sheetData>
@@ -3823,7 +3823,7 @@
         <v>2010</v>
       </c>
       <c r="B2">
-        <v>0.3352</v>
+        <v>0.34815200000000002</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -3831,7 +3831,7 @@
         <v>2011</v>
       </c>
       <c r="B3">
-        <v>0.3352</v>
+        <v>0.34815200000000002</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3839,7 +3839,7 @@
         <v>2012</v>
       </c>
       <c r="B4">
-        <v>0.35489999999999999</v>
+        <v>0.38269999999999998</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -3847,7 +3847,7 @@
         <v>2013</v>
       </c>
       <c r="B5">
-        <v>0.33160000000000001</v>
+        <v>0.35855999999999999</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -3855,7 +3855,7 @@
         <v>2014</v>
       </c>
       <c r="B6">
-        <v>0.31609999999999999</v>
+        <v>0.34620200000000001</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -3863,7 +3863,7 @@
         <v>2015</v>
       </c>
       <c r="B7">
-        <v>0.3337</v>
+        <v>0.36657099999999998</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -3871,7 +3871,7 @@
         <v>2016</v>
       </c>
       <c r="B8">
-        <v>0.3387</v>
+        <v>0.36750899999999997</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -3879,7 +3879,7 @@
         <v>2017</v>
       </c>
       <c r="B9">
-        <v>0.34079999999999999</v>
+        <v>0.36946400000000001</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -3887,7 +3887,7 @@
         <v>2018</v>
       </c>
       <c r="B10">
-        <v>0.34260000000000002</v>
+        <v>0.36212800000000001</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -3895,7 +3895,7 @@
         <v>2019</v>
       </c>
       <c r="B11">
-        <v>0.34989999999999999</v>
+        <v>0.35998599999999997</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -3903,7 +3903,7 @@
         <v>2020</v>
       </c>
       <c r="B12">
-        <v>0.33360000000000001</v>
+        <v>0.347271</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -3911,7 +3911,7 @@
         <v>2021</v>
       </c>
       <c r="B13">
-        <v>0.36370000000000002</v>
+        <v>0.38936500000000002</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -3919,7 +3919,7 @@
         <v>2022</v>
       </c>
       <c r="B14">
-        <v>0.38009999999999999</v>
+        <v>0.39210400000000001</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -3927,7 +3927,7 @@
         <v>2023</v>
       </c>
       <c r="B15">
-        <v>0.38779999999999998</v>
+        <v>0.40636100000000003</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed inSchoolAlignment and Integrated Education Tests -added Education testing into `PersonTest.java` -added appropriate resetting of `eduLeaveSchoolFlag` and `eduExitSampleFlag` -inSchoolAlignment was missing the necessary student share targets (they're now added into `policy parameters.xlsx`) -updated `time_series_factor.xlsx` to include "UK_students_adjustment" -aaded resetting of the `eduLeaveSchoolFlag` into `leavingSchool()` -added updated of the `eduExitSampleFlag`
</commit_message>
<xml_diff>
--- a/input/policy parameters.xlsx
+++ b/input/policy parameters.xlsx
@@ -1,25 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyFiles\99 DEV ENV\JAS-MINE\SimPaths\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pineapple/IdeaProjects/SimPathsUK_refactored/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C55D118-45C5-4278-B5B4-5D567E3F435B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64826849-88D6-0F40-8795-30A440312B2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{E29F3EB7-07F0-4B2F-ABCD-03E4363B7DD7}"/>
+    <workbookView xWindow="22160" yWindow="500" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{E29F3EB7-07F0-4B2F-ABCD-03E4363B7DD7}"/>
   </bookViews>
   <sheets>
     <sheet name="info" sheetId="2" r:id="rId1"/>
     <sheet name="social care" sheetId="1" r:id="rId2"/>
     <sheet name="partnership" sheetId="4" r:id="rId3"/>
-    <sheet name="employment_smales" sheetId="5" r:id="rId4"/>
-    <sheet name="employment_sfemales" sheetId="6" r:id="rId5"/>
-    <sheet name="employment_couples" sheetId="7" r:id="rId6"/>
-    <sheet name="raw data" sheetId="3" r:id="rId7"/>
+    <sheet name="students" sheetId="8" r:id="rId4"/>
+    <sheet name="employment_smales" sheetId="5" r:id="rId5"/>
+    <sheet name="employment_sfemales" sheetId="6" r:id="rId6"/>
+    <sheet name="employment_couples" sheetId="7" r:id="rId7"/>
+    <sheet name="raw data" sheetId="3" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="44">
   <si>
     <t>CAPITAL LIMITS</t>
   </si>
@@ -168,6 +169,12 @@
   </si>
   <si>
     <t>Implied proportion of responsible adults in cohabiting relationship</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Share</t>
   </si>
 </sst>
 </file>
@@ -212,11 +219,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -532,13 +538,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95F81ED4-EE1A-4486-BAEC-BC92A19478AC}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" customWidth="1"/>
+    <col min="1" max="1" width="13.5" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -546,7 +552,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -554,7 +560,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -562,7 +568,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -570,7 +576,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -581,17 +587,17 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="C7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="C8" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
         <v>38</v>
       </c>
@@ -607,9 +613,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5A30919-82CE-4DA6-A5C0-32D0B4E57BD6}">
   <dimension ref="A1:K16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>23</v>
       </c>
@@ -638,7 +644,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>2015</v>
       </c>
@@ -667,7 +673,7 @@
         <v>23250</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2016</v>
       </c>
@@ -696,7 +702,7 @@
         <v>23088.381330685203</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2017</v>
       </c>
@@ -726,7 +732,7 @@
       </c>
       <c r="K4" s="1"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2018</v>
       </c>
@@ -756,7 +762,7 @@
       </c>
       <c r="K5" s="1"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>2019</v>
       </c>
@@ -786,7 +792,7 @@
       </c>
       <c r="K6" s="1"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>2020</v>
       </c>
@@ -816,7 +822,7 @@
       </c>
       <c r="K7" s="1"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>2021</v>
       </c>
@@ -846,7 +852,7 @@
       </c>
       <c r="K8" s="1"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>2022</v>
       </c>
@@ -876,7 +882,7 @@
       </c>
       <c r="K9" s="1"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>2023</v>
       </c>
@@ -906,7 +912,7 @@
       </c>
       <c r="K10" s="1"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>2024</v>
       </c>
@@ -936,7 +942,7 @@
       </c>
       <c r="K11" s="1"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>2025</v>
       </c>
@@ -966,7 +972,7 @@
       </c>
       <c r="K12" s="1"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>2026</v>
       </c>
@@ -996,7 +1002,7 @@
       </c>
       <c r="K13" s="1"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>2027</v>
       </c>
@@ -1026,10 +1032,10 @@
       </c>
       <c r="K14" s="1"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="K15" s="1"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="K16" s="1"/>
     </row>
   </sheetData>
@@ -1040,9 +1046,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8252C88-1FFA-4D3B-9F14-2D9286827575}">
   <dimension ref="A1:B31"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>23</v>
       </c>
@@ -1050,231 +1056,231 @@
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2">
         <v>1994</v>
       </c>
       <c r="B2">
         <v>0.6613654059472992</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3">
         <v>1995</v>
       </c>
       <c r="B3">
         <v>0.65666662435166534</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4">
         <v>1996</v>
       </c>
       <c r="B4">
         <v>0.65162882226991414</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5">
         <v>1997</v>
       </c>
       <c r="B5">
         <v>0.64942413470967808</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6">
         <v>1998</v>
       </c>
       <c r="B6">
         <v>0.64547705146902756</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7">
         <v>1999</v>
       </c>
       <c r="B7">
         <v>0.64460168570888343</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8">
         <v>2000</v>
       </c>
       <c r="B8">
         <v>0.64477324955863657</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9">
         <v>2001</v>
       </c>
       <c r="B9">
         <v>0.64570195231543648</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10">
         <v>2002</v>
       </c>
       <c r="B10">
         <v>0.64737782355652385</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11">
         <v>2003</v>
       </c>
       <c r="B11">
         <v>0.64448143654604106</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12">
         <v>2004</v>
       </c>
       <c r="B12">
         <v>0.64389807700679014</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13">
         <v>2005</v>
       </c>
       <c r="B13">
         <v>0.63601678163112885</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14">
         <v>2006</v>
       </c>
       <c r="B14">
         <v>0.63885715724636716</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15">
         <v>2007</v>
       </c>
       <c r="B15">
         <v>0.63970331929393809</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16">
         <v>2008</v>
       </c>
       <c r="B16">
         <v>0.63745385907812036</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17">
         <v>2009</v>
       </c>
       <c r="B17">
         <v>0.64638142900294271</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18">
         <v>2010</v>
       </c>
       <c r="B18">
         <v>0.64291910814000863</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19">
         <v>2011</v>
       </c>
       <c r="B19">
         <v>0.64183543445918845</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20">
         <v>2012</v>
       </c>
       <c r="B20">
         <v>0.64457311813040019</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21">
         <v>2013</v>
       </c>
       <c r="B21">
         <v>0.64501821298769013</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22">
         <v>2014</v>
       </c>
       <c r="B22">
         <v>0.64303300577959377</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23">
         <v>2015</v>
       </c>
       <c r="B23">
         <v>0.64350137796521267</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="3">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24">
         <v>2016</v>
       </c>
       <c r="B24">
         <v>0.64443090532156433</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="3">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25">
         <v>2017</v>
       </c>
       <c r="B25">
         <v>0.64369538754708922</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="3">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26">
         <v>2018</v>
       </c>
       <c r="B26">
         <v>0.64389678969687036</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" s="3">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27">
         <v>2019</v>
       </c>
       <c r="B27">
         <v>0.63975244582712099</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="3">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28">
         <v>2020</v>
       </c>
       <c r="B28">
         <v>0.64948824720523413</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="3">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29">
         <v>2021</v>
       </c>
       <c r="B29">
         <v>0.64443733677754689</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>2022</v>
       </c>
@@ -1282,7 +1288,7 @@
         <v>0.64425404141077236</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>2023</v>
       </c>
@@ -1296,160 +1302,224 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C02B2D7-F4EC-4D40-840B-FB6BA99B9F2B}">
-  <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9555994B-88C9-EC4A-9208-8AD6657F55B1}">
+  <dimension ref="A1:B27"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="B1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>2010</v>
       </c>
       <c r="B2">
-        <v>0.53940549999999998</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.23899999999999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2011</v>
       </c>
       <c r="B3">
-        <v>0.54004809999999992</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.23899999999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2012</v>
       </c>
       <c r="B4">
-        <v>0.55193539999999996</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.23400000000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2013</v>
       </c>
       <c r="B5">
-        <v>0.57619909999999996</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>2014</v>
       </c>
       <c r="B6">
-        <v>0.57942509999999992</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.22600000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>2015</v>
       </c>
       <c r="B7">
-        <v>0.57820819999999995</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.219</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>2016</v>
       </c>
       <c r="B8">
-        <v>0.57820819999999995</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.218</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>2017</v>
       </c>
       <c r="B9">
-        <v>0.57820819999999995</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.21299999999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>2018</v>
       </c>
       <c r="B10">
-        <v>0.57820819999999995</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>2019</v>
       </c>
       <c r="B11">
-        <v>0.57820819999999995</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.20499999999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>2020</v>
       </c>
       <c r="B12">
-        <v>0.57820819999999995</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.20399999999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>2021</v>
       </c>
       <c r="B13">
-        <v>0.57820819999999995</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.19700000000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>2022</v>
       </c>
       <c r="B14">
-        <v>0.57820819999999995</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.19500000000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>2023</v>
       </c>
       <c r="B15">
-        <v>0.57820819999999995</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.188</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>2024</v>
       </c>
       <c r="B16">
-        <v>0.57820819999999995</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.188</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>2025</v>
       </c>
       <c r="B17">
-        <v>0.57820819999999995</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.188</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>2026</v>
       </c>
       <c r="B18">
-        <v>0.57820819999999995</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.188</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>2027</v>
       </c>
       <c r="B19">
-        <v>0.57820819999999995</v>
+        <v>0.188</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>2028</v>
+      </c>
+      <c r="B20">
+        <v>0.188</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>2029</v>
+      </c>
+      <c r="B21">
+        <v>0.188</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>2030</v>
+      </c>
+      <c r="B22">
+        <v>0.188</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>2031</v>
+      </c>
+      <c r="B23">
+        <v>0.188</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24">
+        <v>2032</v>
+      </c>
+      <c r="B24">
+        <v>0.188</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>2033</v>
+      </c>
+      <c r="B25">
+        <v>0.188</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26">
+        <v>2034</v>
+      </c>
+      <c r="B26">
+        <v>0.188</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>2035</v>
+      </c>
+      <c r="B27">
+        <v>0.188</v>
       </c>
     </row>
   </sheetData>
@@ -1458,11 +1528,11 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2ADCB18-5B9A-4019-89E5-BA38EA9BE54A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C02B2D7-F4EC-4D40-840B-FB6BA99B9F2B}">
   <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>23</v>
       </c>
@@ -1470,148 +1540,148 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>2010</v>
       </c>
       <c r="B2">
-        <v>0.39165939999999999</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.53940549999999998</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2011</v>
       </c>
       <c r="B3">
-        <v>0.40846290000000002</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.54004809999999992</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2012</v>
       </c>
       <c r="B4">
-        <v>0.41123969999999999</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.55193539999999996</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2013</v>
       </c>
       <c r="B5">
-        <v>0.43660460000000001</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.57619909999999996</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>2014</v>
       </c>
       <c r="B6">
-        <v>0.44596649999999999</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.57942509999999992</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>2015</v>
       </c>
       <c r="B7">
-        <v>0.45383590000000001</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.57820819999999995</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>2016</v>
       </c>
       <c r="B8">
-        <v>0.45383590000000001</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.57820819999999995</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>2017</v>
       </c>
       <c r="B9">
-        <v>0.45383590000000001</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.57820819999999995</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>2018</v>
       </c>
       <c r="B10">
-        <v>0.45383590000000001</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.57820819999999995</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>2019</v>
       </c>
       <c r="B11">
-        <v>0.45383590000000001</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.57820819999999995</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>2020</v>
       </c>
       <c r="B12">
-        <v>0.45383590000000001</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.57820819999999995</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>2021</v>
       </c>
       <c r="B13">
-        <v>0.45383590000000001</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.57820819999999995</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>2022</v>
       </c>
       <c r="B14">
-        <v>0.45383590000000001</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.57820819999999995</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>2023</v>
       </c>
       <c r="B15">
-        <v>0.45383590000000001</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.57820819999999995</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>2024</v>
       </c>
       <c r="B16">
-        <v>0.45383590000000001</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.57820819999999995</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>2025</v>
       </c>
       <c r="B17">
-        <v>0.45383590000000001</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.57820819999999995</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>2026</v>
       </c>
       <c r="B18">
-        <v>0.45383590000000001</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.57820819999999995</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>2027</v>
       </c>
       <c r="B19">
-        <v>0.45383590000000001</v>
+        <v>0.57820819999999995</v>
       </c>
     </row>
   </sheetData>
@@ -1620,11 +1690,11 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D244153-91CD-4DE3-A3BE-886BB7506357}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2ADCB18-5B9A-4019-89E5-BA38EA9BE54A}">
   <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>23</v>
       </c>
@@ -1632,148 +1702,148 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>2010</v>
       </c>
       <c r="B2">
-        <v>0.71755429999999998</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.39165939999999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2011</v>
       </c>
       <c r="B3">
-        <v>0.73036599999999996</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.40846290000000002</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2012</v>
       </c>
       <c r="B4">
-        <v>0.74233179999999999</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.41123969999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2013</v>
       </c>
       <c r="B5">
-        <v>0.74778829999999996</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.43660460000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>2014</v>
       </c>
       <c r="B6">
-        <v>0.74564959999999991</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.44596649999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>2015</v>
       </c>
       <c r="B7">
-        <v>0.74624679999999999</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.45383590000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>2016</v>
       </c>
       <c r="B8">
-        <v>0.74345260000000002</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.45383590000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>2017</v>
       </c>
       <c r="B9">
-        <v>0.74345260000000002</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.45383590000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>2018</v>
       </c>
       <c r="B10">
-        <v>0.74345260000000002</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.45383590000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>2019</v>
       </c>
       <c r="B11">
-        <v>0.74345260000000002</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.45383590000000001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>2020</v>
       </c>
       <c r="B12">
-        <v>0.74345260000000002</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.45383590000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>2021</v>
       </c>
       <c r="B13">
-        <v>0.74345260000000002</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.45383590000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>2022</v>
       </c>
       <c r="B14">
-        <v>0.74345260000000002</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.45383590000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>2023</v>
       </c>
       <c r="B15">
-        <v>0.74345260000000002</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.45383590000000001</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>2024</v>
       </c>
       <c r="B16">
-        <v>0.74345260000000002</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.45383590000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>2025</v>
       </c>
       <c r="B17">
-        <v>0.74345260000000002</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.45383590000000001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>2026</v>
       </c>
       <c r="B18">
-        <v>0.74345260000000002</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.45383590000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>2027</v>
       </c>
       <c r="B19">
-        <v>0.74345260000000002</v>
+        <v>0.45383590000000001</v>
       </c>
     </row>
   </sheetData>
@@ -1782,14 +1852,176 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D244153-91CD-4DE3-A3BE-886BB7506357}">
+  <dimension ref="A1:B19"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>2010</v>
+      </c>
+      <c r="B2">
+        <v>0.71755429999999998</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2011</v>
+      </c>
+      <c r="B3">
+        <v>0.73036599999999996</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>2012</v>
+      </c>
+      <c r="B4">
+        <v>0.74233179999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>2013</v>
+      </c>
+      <c r="B5">
+        <v>0.74778829999999996</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>2014</v>
+      </c>
+      <c r="B6">
+        <v>0.74564959999999991</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>2015</v>
+      </c>
+      <c r="B7">
+        <v>0.74624679999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>2016</v>
+      </c>
+      <c r="B8">
+        <v>0.74345260000000002</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>2017</v>
+      </c>
+      <c r="B9">
+        <v>0.74345260000000002</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>2018</v>
+      </c>
+      <c r="B10">
+        <v>0.74345260000000002</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>2019</v>
+      </c>
+      <c r="B11">
+        <v>0.74345260000000002</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>2020</v>
+      </c>
+      <c r="B12">
+        <v>0.74345260000000002</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>2021</v>
+      </c>
+      <c r="B13">
+        <v>0.74345260000000002</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>2022</v>
+      </c>
+      <c r="B14">
+        <v>0.74345260000000002</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>2023</v>
+      </c>
+      <c r="B15">
+        <v>0.74345260000000002</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>2024</v>
+      </c>
+      <c r="B16">
+        <v>0.74345260000000002</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>2025</v>
+      </c>
+      <c r="B17">
+        <v>0.74345260000000002</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>2026</v>
+      </c>
+      <c r="B18">
+        <v>0.74345260000000002</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>2027</v>
+      </c>
+      <c r="B19">
+        <v>0.74345260000000002</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA85A294-76F0-4023-B97D-1E7832E0E774}">
-  <dimension ref="A1:Z33"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:Y33"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="23" max="26" width="9.140625" style="3"/>
+    <col min="23" max="26" width="9.1640625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>34</v>
       </c>
@@ -1800,7 +2032,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>1</v>
       </c>
@@ -1816,7 +2048,7 @@
       <c r="T2" s="2"/>
       <c r="U2" s="2"/>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
         <v>2</v>
       </c>
@@ -1865,14 +2097,14 @@
       <c r="U3" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="X3" s="3" t="s">
+      <c r="X3" t="s">
         <v>40</v>
       </c>
-      <c r="Y3" s="3" t="s">
+      <c r="Y3" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2015</v>
       </c>
@@ -1939,18 +2171,18 @@
         <f t="shared" si="0"/>
         <v>23250</v>
       </c>
-      <c r="W4" s="3">
+      <c r="W4">
         <v>1994</v>
       </c>
-      <c r="X4" s="3">
+      <c r="X4">
         <v>0.49405969999999999</v>
       </c>
-      <c r="Y4" s="3">
+      <c r="Y4">
         <f>2*X4/(2*X4+(1-X4))</f>
         <v>0.6613654059472992</v>
       </c>
     </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2016</v>
       </c>
@@ -2017,19 +2249,19 @@
         <f t="shared" ref="U5:U12" si="9">I5*$K$4/$K5</f>
         <v>23088.381330685203</v>
       </c>
-      <c r="W5" s="3">
+      <c r="W5">
         <f>W4+1</f>
         <v>1995</v>
       </c>
-      <c r="X5" s="3">
+      <c r="X5">
         <v>0.48883369999999998</v>
       </c>
-      <c r="Y5" s="3">
+      <c r="Y5">
         <f t="shared" ref="Y5:Y31" si="10">2*X5/(2*X5+(1-X5))</f>
         <v>0.65666662435166534</v>
       </c>
     </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>2017</v>
       </c>
@@ -2096,19 +2328,19 @@
         <f t="shared" si="9"/>
         <v>22485.493230174081</v>
       </c>
-      <c r="W6" s="3">
-        <f t="shared" ref="W6:W42" si="11">W5+1</f>
+      <c r="W6">
+        <f t="shared" ref="W6:W31" si="11">W5+1</f>
         <v>1996</v>
       </c>
-      <c r="X6" s="3">
+      <c r="X6">
         <v>0.48327110000000001</v>
       </c>
-      <c r="Y6" s="3">
+      <c r="Y6">
         <f t="shared" si="10"/>
         <v>0.65162882226991414</v>
       </c>
     </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>2018</v>
       </c>
@@ -2175,19 +2407,19 @@
         <f t="shared" si="9"/>
         <v>21954.67422096317</v>
       </c>
-      <c r="W7" s="3">
+      <c r="W7">
         <f t="shared" si="11"/>
         <v>1997</v>
       </c>
-      <c r="X7" s="3">
+      <c r="X7">
         <v>0.48084979999999999</v>
       </c>
-      <c r="Y7" s="3">
+      <c r="Y7">
         <f t="shared" si="10"/>
         <v>0.64942413470967808</v>
       </c>
     </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>2019</v>
       </c>
@@ -2254,19 +2486,19 @@
         <f t="shared" si="9"/>
         <v>21567.717996289426</v>
       </c>
-      <c r="W8" s="3">
+      <c r="W8">
         <f t="shared" si="11"/>
         <v>1998</v>
       </c>
-      <c r="X8" s="3">
+      <c r="X8">
         <v>0.47653459999999997</v>
       </c>
-      <c r="Y8" s="3">
+      <c r="Y8">
         <f t="shared" si="10"/>
         <v>0.64547705146902756</v>
       </c>
     </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>2020</v>
       </c>
@@ -2333,19 +2565,19 @@
         <f t="shared" si="9"/>
         <v>21389.144434222631</v>
       </c>
-      <c r="W9" s="3">
+      <c r="W9">
         <f t="shared" si="11"/>
         <v>1999</v>
       </c>
-      <c r="X9" s="3">
+      <c r="X9">
         <v>0.47558099999999998</v>
       </c>
-      <c r="Y9" s="3">
+      <c r="Y9">
         <f t="shared" si="10"/>
         <v>0.64460168570888343</v>
       </c>
     </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>2021</v>
       </c>
@@ -2412,19 +2644,19 @@
         <f t="shared" si="9"/>
         <v>20833.333333333336</v>
       </c>
-      <c r="W10" s="3">
+      <c r="W10">
         <f t="shared" si="11"/>
         <v>2000</v>
       </c>
-      <c r="X10" s="3">
+      <c r="X10">
         <v>0.47576780000000002</v>
       </c>
-      <c r="Y10" s="3">
+      <c r="Y10">
         <f t="shared" si="10"/>
         <v>0.64477324955863657</v>
       </c>
     </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>2022</v>
       </c>
@@ -2491,19 +2723,19 @@
         <f t="shared" si="9"/>
         <v>19104.354971240755</v>
       </c>
-      <c r="W11" s="3">
+      <c r="W11">
         <f t="shared" si="11"/>
         <v>2001</v>
       </c>
-      <c r="X11" s="3">
+      <c r="X11">
         <v>0.47677979999999998</v>
       </c>
-      <c r="Y11" s="3">
+      <c r="Y11">
         <f t="shared" si="10"/>
         <v>0.64570195231543648</v>
       </c>
     </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>2023</v>
       </c>
@@ -2570,19 +2802,19 @@
         <f t="shared" si="9"/>
         <v>18663.611748853393</v>
       </c>
-      <c r="W12" s="3">
+      <c r="W12">
         <f t="shared" si="11"/>
         <v>2002</v>
       </c>
-      <c r="X12" s="3">
+      <c r="X12">
         <v>0.47860950000000002</v>
       </c>
-      <c r="Y12" s="3">
+      <c r="Y12">
         <f t="shared" si="10"/>
         <v>0.64737782355652385</v>
       </c>
     </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>2024</v>
       </c>
@@ -2631,19 +2863,19 @@
         <f t="shared" ref="U13:U16" si="14">I13*$K$4/$K13</f>
         <v>18360.484915871581</v>
       </c>
-      <c r="W13" s="3">
+      <c r="W13">
         <f t="shared" si="11"/>
         <v>2003</v>
       </c>
-      <c r="X13" s="3">
+      <c r="X13">
         <v>0.47545009999999999</v>
       </c>
-      <c r="Y13" s="3">
+      <c r="Y13">
         <f t="shared" si="10"/>
         <v>0.64448143654604106</v>
       </c>
     </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>2025</v>
       </c>
@@ -2692,19 +2924,19 @@
         <f t="shared" si="14"/>
         <v>18006.917277302477</v>
       </c>
-      <c r="W14" s="3">
+      <c r="W14">
         <f t="shared" si="11"/>
         <v>2004</v>
       </c>
-      <c r="X14" s="3">
+      <c r="X14">
         <v>0.4748154</v>
       </c>
-      <c r="Y14" s="3">
+      <c r="Y14">
         <f t="shared" si="10"/>
         <v>0.64389807700679014</v>
       </c>
     </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>2026</v>
       </c>
@@ -2753,19 +2985,19 @@
         <f t="shared" si="14"/>
         <v>17653.840467943606</v>
       </c>
-      <c r="W15" s="3">
+      <c r="W15">
         <f t="shared" si="11"/>
         <v>2005</v>
       </c>
-      <c r="X15" s="3">
+      <c r="X15">
         <v>0.46629369999999998</v>
       </c>
-      <c r="Y15" s="3">
+      <c r="Y15">
         <f t="shared" si="10"/>
         <v>0.63601678163112885</v>
       </c>
     </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>2027</v>
       </c>
@@ -2814,227 +3046,227 @@
         <f t="shared" si="14"/>
         <v>17205.948416783383</v>
       </c>
-      <c r="W16" s="3">
+      <c r="W16">
         <f t="shared" si="11"/>
         <v>2006</v>
       </c>
-      <c r="X16" s="3">
+      <c r="X16">
         <v>0.46935349999999998</v>
       </c>
-      <c r="Y16" s="3">
+      <c r="Y16">
         <f t="shared" si="10"/>
         <v>0.63885715724636716</v>
       </c>
     </row>
-    <row r="17" spans="23:25" x14ac:dyDescent="0.25">
-      <c r="W17" s="3">
+    <row r="17" spans="23:25" x14ac:dyDescent="0.2">
+      <c r="W17">
         <f t="shared" si="11"/>
         <v>2007</v>
       </c>
-      <c r="X17" s="3">
+      <c r="X17">
         <v>0.4702675</v>
       </c>
-      <c r="Y17" s="3">
+      <c r="Y17">
         <f t="shared" si="10"/>
         <v>0.63970331929393809</v>
       </c>
     </row>
-    <row r="18" spans="23:25" x14ac:dyDescent="0.25">
-      <c r="W18" s="3">
+    <row r="18" spans="23:25" x14ac:dyDescent="0.2">
+      <c r="W18">
         <f t="shared" si="11"/>
         <v>2008</v>
       </c>
-      <c r="X18" s="3">
+      <c r="X18">
         <v>0.46784019999999998</v>
       </c>
-      <c r="Y18" s="3">
+      <c r="Y18">
         <f t="shared" si="10"/>
         <v>0.63745385907812036</v>
       </c>
     </row>
-    <row r="19" spans="23:25" x14ac:dyDescent="0.25">
-      <c r="W19" s="3">
+    <row r="19" spans="23:25" x14ac:dyDescent="0.2">
+      <c r="W19">
         <f t="shared" si="11"/>
         <v>2009</v>
       </c>
-      <c r="X19" s="3">
+      <c r="X19">
         <v>0.47752109999999998</v>
       </c>
-      <c r="Y19" s="3">
+      <c r="Y19">
         <f t="shared" si="10"/>
         <v>0.64638142900294271</v>
       </c>
     </row>
-    <row r="20" spans="23:25" x14ac:dyDescent="0.25">
-      <c r="W20" s="3">
+    <row r="20" spans="23:25" x14ac:dyDescent="0.2">
+      <c r="W20">
         <f t="shared" si="11"/>
         <v>2010</v>
       </c>
-      <c r="X20" s="3">
+      <c r="X20">
         <v>0.47375149999999999</v>
       </c>
-      <c r="Y20" s="3">
+      <c r="Y20">
         <f t="shared" si="10"/>
         <v>0.64291910814000863</v>
       </c>
     </row>
-    <row r="21" spans="23:25" x14ac:dyDescent="0.25">
-      <c r="W21" s="3">
+    <row r="21" spans="23:25" x14ac:dyDescent="0.2">
+      <c r="W21">
         <f t="shared" si="11"/>
         <v>2011</v>
       </c>
-      <c r="X21" s="3">
+      <c r="X21">
         <v>0.47257559999999998</v>
       </c>
-      <c r="Y21" s="3">
+      <c r="Y21">
         <f t="shared" si="10"/>
         <v>0.64183543445918845</v>
       </c>
     </row>
-    <row r="22" spans="23:25" x14ac:dyDescent="0.25">
-      <c r="W22" s="3">
+    <row r="22" spans="23:25" x14ac:dyDescent="0.2">
+      <c r="W22">
         <f t="shared" si="11"/>
         <v>2012</v>
       </c>
-      <c r="X22" s="3">
+      <c r="X22">
         <v>0.47554990000000003</v>
       </c>
-      <c r="Y22" s="3">
+      <c r="Y22">
         <f t="shared" si="10"/>
         <v>0.64457311813040019</v>
       </c>
     </row>
-    <row r="23" spans="23:25" x14ac:dyDescent="0.25">
-      <c r="W23" s="3">
+    <row r="23" spans="23:25" x14ac:dyDescent="0.2">
+      <c r="W23">
         <f t="shared" si="11"/>
         <v>2013</v>
       </c>
-      <c r="X23" s="3">
+      <c r="X23">
         <v>0.47603459999999997</v>
       </c>
-      <c r="Y23" s="3">
+      <c r="Y23">
         <f t="shared" si="10"/>
         <v>0.64501821298769013</v>
       </c>
     </row>
-    <row r="24" spans="23:25" x14ac:dyDescent="0.25">
-      <c r="W24" s="3">
+    <row r="24" spans="23:25" x14ac:dyDescent="0.2">
+      <c r="W24">
         <f t="shared" si="11"/>
         <v>2014</v>
       </c>
-      <c r="X24" s="3">
+      <c r="X24">
         <v>0.4738752</v>
       </c>
-      <c r="Y24" s="3">
+      <c r="Y24">
         <f t="shared" si="10"/>
         <v>0.64303300577959377</v>
       </c>
     </row>
-    <row r="25" spans="23:25" x14ac:dyDescent="0.25">
-      <c r="W25" s="3">
+    <row r="25" spans="23:25" x14ac:dyDescent="0.2">
+      <c r="W25">
         <f t="shared" si="11"/>
         <v>2015</v>
       </c>
-      <c r="X25" s="3">
+      <c r="X25">
         <v>0.47438409999999998</v>
       </c>
-      <c r="Y25" s="3">
+      <c r="Y25">
         <f t="shared" si="10"/>
         <v>0.64350137796521267</v>
       </c>
     </row>
-    <row r="26" spans="23:25" x14ac:dyDescent="0.25">
-      <c r="W26" s="3">
+    <row r="26" spans="23:25" x14ac:dyDescent="0.2">
+      <c r="W26">
         <f t="shared" si="11"/>
         <v>2016</v>
       </c>
-      <c r="X26" s="3">
+      <c r="X26">
         <v>0.47539510000000001</v>
       </c>
-      <c r="Y26" s="3">
+      <c r="Y26">
         <f t="shared" si="10"/>
         <v>0.64443090532156433</v>
       </c>
     </row>
-    <row r="27" spans="23:25" x14ac:dyDescent="0.25">
-      <c r="W27" s="3">
+    <row r="27" spans="23:25" x14ac:dyDescent="0.2">
+      <c r="W27">
         <f t="shared" si="11"/>
         <v>2017</v>
       </c>
-      <c r="X27" s="3">
+      <c r="X27">
         <v>0.47459499999999999</v>
       </c>
-      <c r="Y27" s="3">
+      <c r="Y27">
         <f t="shared" si="10"/>
         <v>0.64369538754708922</v>
       </c>
     </row>
-    <row r="28" spans="23:25" x14ac:dyDescent="0.25">
-      <c r="W28" s="3">
+    <row r="28" spans="23:25" x14ac:dyDescent="0.2">
+      <c r="W28">
         <f t="shared" si="11"/>
         <v>2018</v>
       </c>
-      <c r="X28" s="3">
+      <c r="X28">
         <v>0.47481400000000001</v>
       </c>
-      <c r="Y28" s="3">
+      <c r="Y28">
         <f t="shared" si="10"/>
         <v>0.64389678969687036</v>
       </c>
     </row>
-    <row r="29" spans="23:25" x14ac:dyDescent="0.25">
-      <c r="W29" s="3">
+    <row r="29" spans="23:25" x14ac:dyDescent="0.2">
+      <c r="W29">
         <f t="shared" si="11"/>
         <v>2019</v>
       </c>
-      <c r="X29" s="3">
+      <c r="X29">
         <v>0.47032059999999998</v>
       </c>
-      <c r="Y29" s="3">
+      <c r="Y29">
         <f t="shared" si="10"/>
         <v>0.63975244582712099</v>
       </c>
     </row>
-    <row r="30" spans="23:25" x14ac:dyDescent="0.25">
-      <c r="W30" s="3">
+    <row r="30" spans="23:25" x14ac:dyDescent="0.2">
+      <c r="W30">
         <f t="shared" si="11"/>
         <v>2020</v>
       </c>
-      <c r="X30" s="3">
+      <c r="X30">
         <v>0.48092010000000002</v>
       </c>
-      <c r="Y30" s="3">
+      <c r="Y30">
         <f t="shared" si="10"/>
         <v>0.64948824720523413</v>
       </c>
     </row>
-    <row r="31" spans="23:25" x14ac:dyDescent="0.25">
-      <c r="W31" s="3">
+    <row r="31" spans="23:25" x14ac:dyDescent="0.2">
+      <c r="W31">
         <f t="shared" si="11"/>
         <v>2021</v>
       </c>
-      <c r="X31" s="3">
+      <c r="X31">
         <v>0.47540209999999999</v>
       </c>
-      <c r="Y31" s="3">
+      <c r="Y31">
         <f t="shared" si="10"/>
         <v>0.64443733677754689</v>
       </c>
     </row>
-    <row r="32" spans="23:25" x14ac:dyDescent="0.25">
-      <c r="W32" s="3">
+    <row r="32" spans="23:25" x14ac:dyDescent="0.2">
+      <c r="W32">
         <v>2022</v>
       </c>
-      <c r="Y32" s="3">
+      <c r="Y32">
         <f>AVERAGE(Y27:Y31)</f>
         <v>0.64425404141077236</v>
       </c>
     </row>
-    <row r="33" spans="23:25" x14ac:dyDescent="0.25">
-      <c r="W33" s="3">
+    <row r="33" spans="23:25" x14ac:dyDescent="0.2">
+      <c r="W33">
         <v>2023</v>
       </c>
-      <c r="Y33" s="3">
+      <c r="Y33">
         <f>Y32</f>
         <v>0.64425404141077236</v>
       </c>

</xml_diff>

<commit_message>
Updated inSchool Alignment targets
</commit_message>
<xml_diff>
--- a/input/policy parameters.xlsx
+++ b/input/policy parameters.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pineapple/IdeaProjects/SimPathsUK_refactored/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64826849-88D6-0F40-8795-30A440312B2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{690D1327-0781-FC43-BD2F-983FDD87B78E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22160" yWindow="500" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{E29F3EB7-07F0-4B2F-ABCD-03E4363B7DD7}"/>
   </bookViews>
@@ -16,11 +16,10 @@
     <sheet name="info" sheetId="2" r:id="rId1"/>
     <sheet name="social care" sheetId="1" r:id="rId2"/>
     <sheet name="partnership" sheetId="4" r:id="rId3"/>
-    <sheet name="students" sheetId="8" r:id="rId4"/>
-    <sheet name="employment_smales" sheetId="5" r:id="rId5"/>
-    <sheet name="employment_sfemales" sheetId="6" r:id="rId6"/>
-    <sheet name="employment_couples" sheetId="7" r:id="rId7"/>
-    <sheet name="raw data" sheetId="3" r:id="rId8"/>
+    <sheet name="employment_smales" sheetId="5" r:id="rId4"/>
+    <sheet name="employment_sfemales" sheetId="6" r:id="rId5"/>
+    <sheet name="employment_couples" sheetId="7" r:id="rId6"/>
+    <sheet name="raw data" sheetId="3" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="42">
   <si>
     <t>CAPITAL LIMITS</t>
   </si>
@@ -169,12 +168,6 @@
   </si>
   <si>
     <t>Implied proportion of responsible adults in cohabiting relationship</t>
-  </si>
-  <si>
-    <t>Year</t>
-  </si>
-  <si>
-    <t>Share</t>
   </si>
 </sst>
 </file>
@@ -1302,232 +1295,6 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9555994B-88C9-EC4A-9208-8AD6657F55B1}">
-  <dimension ref="A1:B27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>2010</v>
-      </c>
-      <c r="B2">
-        <v>0.23899999999999999</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3">
-        <v>2011</v>
-      </c>
-      <c r="B3">
-        <v>0.23899999999999999</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4">
-        <v>2012</v>
-      </c>
-      <c r="B4">
-        <v>0.23400000000000001</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>2013</v>
-      </c>
-      <c r="B5">
-        <v>0.23</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>2014</v>
-      </c>
-      <c r="B6">
-        <v>0.22600000000000001</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>2015</v>
-      </c>
-      <c r="B7">
-        <v>0.219</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>2016</v>
-      </c>
-      <c r="B8">
-        <v>0.218</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9">
-        <v>2017</v>
-      </c>
-      <c r="B9">
-        <v>0.21299999999999999</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10">
-        <v>2018</v>
-      </c>
-      <c r="B10">
-        <v>0.21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11">
-        <v>2019</v>
-      </c>
-      <c r="B11">
-        <v>0.20499999999999999</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12">
-        <v>2020</v>
-      </c>
-      <c r="B12">
-        <v>0.20399999999999999</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13">
-        <v>2021</v>
-      </c>
-      <c r="B13">
-        <v>0.19700000000000001</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A14">
-        <v>2022</v>
-      </c>
-      <c r="B14">
-        <v>0.19500000000000001</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A15">
-        <v>2023</v>
-      </c>
-      <c r="B15">
-        <v>0.188</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A16">
-        <v>2024</v>
-      </c>
-      <c r="B16">
-        <v>0.188</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17">
-        <v>2025</v>
-      </c>
-      <c r="B17">
-        <v>0.188</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A18">
-        <v>2026</v>
-      </c>
-      <c r="B18">
-        <v>0.188</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19">
-        <v>2027</v>
-      </c>
-      <c r="B19">
-        <v>0.188</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A20">
-        <v>2028</v>
-      </c>
-      <c r="B20">
-        <v>0.188</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A21">
-        <v>2029</v>
-      </c>
-      <c r="B21">
-        <v>0.188</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22">
-        <v>2030</v>
-      </c>
-      <c r="B22">
-        <v>0.188</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A23">
-        <v>2031</v>
-      </c>
-      <c r="B23">
-        <v>0.188</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A24">
-        <v>2032</v>
-      </c>
-      <c r="B24">
-        <v>0.188</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A25">
-        <v>2033</v>
-      </c>
-      <c r="B25">
-        <v>0.188</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A26">
-        <v>2034</v>
-      </c>
-      <c r="B26">
-        <v>0.188</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A27">
-        <v>2035</v>
-      </c>
-      <c r="B27">
-        <v>0.188</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C02B2D7-F4EC-4D40-840B-FB6BA99B9F2B}">
   <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -1689,7 +1456,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2ADCB18-5B9A-4019-89E5-BA38EA9BE54A}">
   <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -1851,7 +1618,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D244153-91CD-4DE3-A3BE-886BB7506357}">
   <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -2013,7 +1780,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA85A294-76F0-4023-B97D-1E7832E0E774}">
   <dimension ref="A1:Y33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>

</xml_diff>